<commit_message>
Update trains and loco export 2026-04-04 18:33:39
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -43384,7 +43384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -43400,49 +43400,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bdca</t>
+          <t>aurizon*</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bnbn</t>
+          <t>bdca</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bnfg</t>
+          <t>bnbn</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bnvl</t>
+          <t>bnfg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>brbr</t>
+          <t>bnvl</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>brcl</t>
+          <t>brbr</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>brfg</t>
+          <t>brcl</t>
         </is>
       </c>
     </row>
@@ -43456,152 +43456,159 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>brip</t>
+          <t>brfg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>brsp</t>
+          <t>brip</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cabd</t>
+          <t>brsp</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>caca</t>
+          <t>cabd</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cadb</t>
+          <t>caca</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>caip</t>
+          <t>cadb</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>clbr</t>
+          <t>caip</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dbca</t>
+          <t>clbr</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dulwich hill line</t>
+          <t>dbca</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>fgbr</t>
+          <t>dulwich hill line</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gcr1</t>
+          <t>fgbr</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gungahlin place - alinga street</t>
+          <t>gcr1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ipbr</t>
+          <t>gungahlin place - alinga street</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>iprw</t>
+          <t>ipbr</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kingsford line</t>
+          <t>iprw</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>metro north west &amp; bankstown line</t>
+          <t>kingsford line</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>newcastle interchange - newcastle beach line service</t>
+          <t>metro north west &amp; bankstown line</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>randwick line</t>
+          <t>newcastle interchange - newcastle beach line service</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>rwip</t>
+          <t>randwick line</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>shcl</t>
+          <t>rwip</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>spbr</t>
+          <t>shcl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
+        <is>
+          <t>spbr</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>vlbn</t>
         </is>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-05 15:56:54
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -4056,7 +4056,11 @@
         </is>
       </c>
       <c r="B215" t="inlineStr"/>
-      <c r="C215" t="inlineStr"/>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>PN Toll Freight</t>
+        </is>
+      </c>
       <c r="D215" t="inlineStr">
         <is>
           <t>2026-04-05 15:26:42</t>
@@ -7399,7 +7403,11 @@
         </is>
       </c>
       <c r="B424" t="inlineStr"/>
-      <c r="C424" t="inlineStr"/>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Aurizon Empty Grain</t>
+        </is>
+      </c>
       <c r="D424" t="inlineStr">
         <is>
           <t>2026-04-05 01:09:16</t>
@@ -7577,7 +7585,11 @@
         </is>
       </c>
       <c r="B435" t="inlineStr"/>
-      <c r="C435" t="inlineStr"/>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Hunter Line Service</t>
+        </is>
+      </c>
       <c r="D435" t="inlineStr">
         <is>
           <t>2026-04-03 15:09:22</t>
@@ -22586,7 +22598,11 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PN Toll Freight</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>2026-04-05 15:26:42</t>
@@ -24916,7 +24932,11 @@
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Aurizon Empty Grain</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
           <t>2026-04-05 01:09:16</t>
@@ -33245,7 +33265,11 @@
         </is>
       </c>
       <c r="B617" t="inlineStr"/>
-      <c r="C617" t="inlineStr"/>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Hunter Line Service</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
           <t>2026-04-03 15:09:22</t>

</xml_diff>

<commit_message>
Update trains and loco database files
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -580,7 +580,7 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Northern Line Service</t>
+          <t>Empty Car Transfer for Maintenance</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1174,7 +1174,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>V/Line Empty Car Transfer</t>
+          <t>Empty Car Transfer for Maintenance</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1228,7 +1228,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>North East BG Line Service</t>
+          <t>North East Line BG Service</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1738,7 +1738,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Northern Line Service</t>
+          <t>South Western Line Service</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2306,7 +2306,7 @@
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>South Western Line Service</t>
+          <t>Northern Line Service</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3494,7 +3494,7 @@
       <c r="B173" t="inlineStr"/>
       <c r="C173" t="inlineStr">
         <is>
-          <t>SSR Shunter</t>
+          <t>SSR Cement Trip Train</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -7520,7 +7520,7 @@
       <c r="B410" t="inlineStr"/>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Aurizon Loaded Grain</t>
+          <t>Aurizon Wagon Transfer</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -8818,7 +8818,7 @@
       <c r="B489" t="inlineStr"/>
       <c r="C489" t="inlineStr">
         <is>
-          <t>SCT Shuttle</t>
+          <t>SCT Intermodal</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -9588,7 +9588,7 @@
       <c r="B533" t="inlineStr"/>
       <c r="C533" t="inlineStr">
         <is>
-          <t>NSW TrainLink Xplorer</t>
+          <t>NSW Trainlink Empty Car Transfer</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -9878,7 +9878,7 @@
       <c r="B550" t="inlineStr"/>
       <c r="C550" t="inlineStr">
         <is>
-          <t>PN Containerised Freight</t>
+          <t>PN Containerised Freight via RRL</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
@@ -10872,7 +10872,7 @@
       <c r="B607" t="inlineStr"/>
       <c r="C607" t="inlineStr">
         <is>
-          <t>Hunter Line Service</t>
+          <t>Hunter Railcar Transfer</t>
         </is>
       </c>
       <c r="D607" t="inlineStr">
@@ -14008,7 +14008,7 @@
       <c r="B785" t="inlineStr"/>
       <c r="C785" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Belgrave Line</t>
         </is>
       </c>
       <c r="D785" t="inlineStr">
@@ -14026,7 +14026,7 @@
       <c r="B786" t="inlineStr"/>
       <c r="C786" t="inlineStr">
         <is>
-          <t>Mernda Line</t>
+          <t>Hurstbridge Line</t>
         </is>
       </c>
       <c r="D786" t="inlineStr">
@@ -14116,7 +14116,7 @@
       <c r="B791" t="inlineStr"/>
       <c r="C791" t="inlineStr">
         <is>
-          <t>Hurstbridge Line</t>
+          <t>Glen Waverley Line</t>
         </is>
       </c>
       <c r="D791" t="inlineStr">
@@ -14710,7 +14710,7 @@
       <c r="B824" t="inlineStr"/>
       <c r="C824" t="inlineStr">
         <is>
-          <t>Mernda Line</t>
+          <t>Hurstbridge Line</t>
         </is>
       </c>
       <c r="D824" t="inlineStr">
@@ -15142,7 +15142,7 @@
       <c r="B848" t="inlineStr"/>
       <c r="C848" t="inlineStr">
         <is>
-          <t>Belgrave Line</t>
+          <t>Lilydale Line</t>
         </is>
       </c>
       <c r="D848" t="inlineStr">
@@ -15466,7 +15466,7 @@
       <c r="B866" t="inlineStr"/>
       <c r="C866" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
@@ -15862,7 +15862,7 @@
       <c r="B888" t="inlineStr"/>
       <c r="C888" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D888" t="inlineStr">
@@ -17208,7 +17208,7 @@
       <c r="B963" t="inlineStr"/>
       <c r="C963" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
@@ -17316,7 +17316,7 @@
       <c r="B969" t="inlineStr"/>
       <c r="C969" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D969" t="inlineStr">
@@ -18036,7 +18036,7 @@
       <c r="B1009" t="inlineStr"/>
       <c r="C1009" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Mernda Line</t>
         </is>
       </c>
       <c r="D1009" t="inlineStr">
@@ -18090,7 +18090,7 @@
       <c r="B1012" t="inlineStr"/>
       <c r="C1012" t="inlineStr">
         <is>
-          <t>Belgrave Line</t>
+          <t>Glen Waverley Line</t>
         </is>
       </c>
       <c r="D1012" t="inlineStr">
@@ -18270,7 +18270,7 @@
       <c r="B1022" t="inlineStr"/>
       <c r="C1022" t="inlineStr">
         <is>
-          <t>Lilydale Line</t>
+          <t>Mernda Line</t>
         </is>
       </c>
       <c r="D1022" t="inlineStr">
@@ -18504,7 +18504,7 @@
       <c r="B1035" t="inlineStr"/>
       <c r="C1035" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Lilydale Line</t>
         </is>
       </c>
       <c r="D1035" t="inlineStr">
@@ -18648,7 +18648,7 @@
       <c r="B1043" t="inlineStr"/>
       <c r="C1043" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1043" t="inlineStr">
@@ -18702,7 +18702,7 @@
       <c r="B1046" t="inlineStr"/>
       <c r="C1046" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1046" t="inlineStr">
@@ -19008,7 +19008,7 @@
       <c r="B1063" t="inlineStr"/>
       <c r="C1063" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1063" t="inlineStr">
@@ -19098,7 +19098,7 @@
       <c r="B1068" t="inlineStr"/>
       <c r="C1068" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1068" t="inlineStr">
@@ -19188,7 +19188,7 @@
       <c r="B1073" t="inlineStr"/>
       <c r="C1073" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D1073" t="inlineStr">
@@ -19242,7 +19242,7 @@
       <c r="B1076" t="inlineStr"/>
       <c r="C1076" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D1076" t="inlineStr">
@@ -19260,7 +19260,7 @@
       <c r="B1077" t="inlineStr"/>
       <c r="C1077" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1077" t="inlineStr">
@@ -19404,7 +19404,7 @@
       <c r="B1085" t="inlineStr"/>
       <c r="C1085" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1085" t="inlineStr">
@@ -19458,7 +19458,7 @@
       <c r="B1088" t="inlineStr"/>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D1088" t="inlineStr">
@@ -19566,7 +19566,7 @@
       <c r="B1094" t="inlineStr"/>
       <c r="C1094" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1094" t="inlineStr">
@@ -19710,7 +19710,7 @@
       <c r="B1102" t="inlineStr"/>
       <c r="C1102" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1102" t="inlineStr">
@@ -19782,7 +19782,7 @@
       <c r="B1106" t="inlineStr"/>
       <c r="C1106" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1106" t="inlineStr">
@@ -22424,7 +22424,7 @@
       <c r="B1263" t="inlineStr"/>
       <c r="C1263" t="inlineStr">
         <is>
-          <t>Aurizon Shunter</t>
+          <t>Aurizon Nickel Residue</t>
         </is>
       </c>
       <c r="D1263" t="inlineStr">
@@ -22956,7 +22956,7 @@
       <c r="B1295" t="inlineStr"/>
       <c r="C1295" t="inlineStr">
         <is>
-          <t>QUBE Container Train</t>
+          <t>QUBE Grain</t>
         </is>
       </c>
       <c r="D1295" t="inlineStr">
@@ -24418,7 +24418,7 @@
       <c r="B1382" t="inlineStr"/>
       <c r="C1382" t="inlineStr">
         <is>
-          <t>South Coast Service</t>
+          <t>Sydney Trains Empty Car Transfer</t>
         </is>
       </c>
       <c r="D1382" t="inlineStr">
@@ -34001,7 +34001,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SCT Shuttle</t>
+          <t>SCT Intermodal</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -37373,7 +37373,7 @@
       <c r="B216" t="inlineStr"/>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -37909,7 +37909,7 @@
       <c r="B246" t="inlineStr"/>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -37927,7 +37927,7 @@
       <c r="B247" t="inlineStr"/>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -38013,7 +38013,7 @@
       <c r="B252" t="inlineStr"/>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Lilydale Line</t>
+          <t>Mernda Line</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -38481,7 +38481,7 @@
       <c r="B278" t="inlineStr"/>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -43849,7 +43849,7 @@
       <c r="B582" t="inlineStr"/>
       <c r="C582" t="inlineStr">
         <is>
-          <t>Mernda Line</t>
+          <t>Hurstbridge Line</t>
         </is>
       </c>
       <c r="D582" t="inlineStr">
@@ -44517,7 +44517,7 @@
       <c r="B620" t="inlineStr"/>
       <c r="C620" t="inlineStr">
         <is>
-          <t>Northern Line Service</t>
+          <t>South Western Line Service</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -44941,7 +44941,7 @@
       <c r="B644" t="inlineStr"/>
       <c r="C644" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
@@ -45049,7 +45049,7 @@
       <c r="B650" t="inlineStr"/>
       <c r="C650" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
@@ -45983,7 +45983,7 @@
       <c r="B703" t="inlineStr"/>
       <c r="C703" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D703" t="inlineStr">
@@ -47623,7 +47623,7 @@
       <c r="B795" t="inlineStr"/>
       <c r="C795" t="inlineStr">
         <is>
-          <t>Mernda Line</t>
+          <t>Hurstbridge Line</t>
         </is>
       </c>
       <c r="D795" t="inlineStr">
@@ -48895,7 +48895,7 @@
       <c r="B867" t="inlineStr"/>
       <c r="C867" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
@@ -49373,7 +49373,7 @@
       <c r="B894" t="inlineStr"/>
       <c r="C894" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Belgrave Line</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
@@ -50161,7 +50161,7 @@
       <c r="B938" t="inlineStr"/>
       <c r="C938" t="inlineStr">
         <is>
-          <t>V/Line Empty Car Transfer</t>
+          <t>Empty Car Transfer for Maintenance</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
@@ -50985,7 +50985,7 @@
       <c r="B984" t="inlineStr"/>
       <c r="C984" t="inlineStr">
         <is>
-          <t>North East BG Line Service</t>
+          <t>North East Line BG Service</t>
         </is>
       </c>
       <c r="D984" t="inlineStr">
@@ -53017,7 +53017,7 @@
       <c r="B1100" t="inlineStr"/>
       <c r="C1100" t="inlineStr">
         <is>
-          <t>QUBE Container Train</t>
+          <t>QUBE Grain</t>
         </is>
       </c>
       <c r="D1100" t="inlineStr">
@@ -54316,7 +54316,7 @@
       <c r="B1173" t="inlineStr"/>
       <c r="C1173" t="inlineStr">
         <is>
-          <t>Cranbourne Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1173" t="inlineStr">
@@ -54514,7 +54514,7 @@
       <c r="B1184" t="inlineStr"/>
       <c r="C1184" t="inlineStr">
         <is>
-          <t>Northern Line Service</t>
+          <t>Empty Car Transfer for Maintenance</t>
         </is>
       </c>
       <c r="D1184" t="inlineStr">
@@ -55241,7 +55241,7 @@
       <c r="B1225" t="inlineStr"/>
       <c r="C1225" t="inlineStr">
         <is>
-          <t>Hurstbridge Line</t>
+          <t>Glen Waverley Line</t>
         </is>
       </c>
       <c r="D1225" t="inlineStr">
@@ -56799,7 +56799,7 @@
       <c r="B1314" t="inlineStr"/>
       <c r="C1314" t="inlineStr">
         <is>
-          <t>South Western Line Service</t>
+          <t>Northern Line Service</t>
         </is>
       </c>
       <c r="D1314" t="inlineStr">
@@ -57443,7 +57443,7 @@
       <c r="B1350" t="inlineStr"/>
       <c r="C1350" t="inlineStr">
         <is>
-          <t>NSW TrainLink Xplorer</t>
+          <t>NSW Trainlink Empty Car Transfer</t>
         </is>
       </c>
       <c r="D1350" t="inlineStr">
@@ -57919,7 +57919,7 @@
       <c r="B1378" t="inlineStr"/>
       <c r="C1378" t="inlineStr">
         <is>
-          <t>Aurizon Loaded Grain</t>
+          <t>Aurizon Wagon Transfer</t>
         </is>
       </c>
       <c r="D1378" t="inlineStr">
@@ -58549,7 +58549,7 @@
       <c r="B1413" t="inlineStr"/>
       <c r="C1413" t="inlineStr">
         <is>
-          <t>PN Containerised Freight</t>
+          <t>PN Containerised Freight via RRL</t>
         </is>
       </c>
       <c r="D1413" t="inlineStr">
@@ -58671,7 +58671,7 @@
       <c r="B1420" t="inlineStr"/>
       <c r="C1420" t="inlineStr">
         <is>
-          <t>Hunter Line Service</t>
+          <t>Hunter Railcar Transfer</t>
         </is>
       </c>
       <c r="D1420" t="inlineStr">
@@ -58937,7 +58937,7 @@
       <c r="B1435" t="inlineStr"/>
       <c r="C1435" t="inlineStr">
         <is>
-          <t>South Coast Service</t>
+          <t>Sydney Trains Empty Car Transfer</t>
         </is>
       </c>
       <c r="D1435" t="inlineStr">
@@ -59757,7 +59757,7 @@
       <c r="B1481" t="inlineStr"/>
       <c r="C1481" t="inlineStr">
         <is>
-          <t>SSR Shunter</t>
+          <t>SSR Cement Trip Train</t>
         </is>
       </c>
       <c r="D1481" t="inlineStr">
@@ -62167,7 +62167,7 @@
       <c r="B1622" t="inlineStr"/>
       <c r="C1622" t="inlineStr">
         <is>
-          <t>Belgrave Line</t>
+          <t>Lilydale Line</t>
         </is>
       </c>
       <c r="D1622" t="inlineStr">
@@ -62725,7 +62725,7 @@
       <c r="B1653" t="inlineStr"/>
       <c r="C1653" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D1653" t="inlineStr">
@@ -62779,7 +62779,7 @@
       <c r="B1656" t="inlineStr"/>
       <c r="C1656" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D1656" t="inlineStr">
@@ -63067,7 +63067,7 @@
       <c r="B1672" t="inlineStr"/>
       <c r="C1672" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Mernda Line</t>
         </is>
       </c>
       <c r="D1672" t="inlineStr">
@@ -63085,7 +63085,7 @@
       <c r="B1673" t="inlineStr"/>
       <c r="C1673" t="inlineStr">
         <is>
-          <t>Belgrave Line</t>
+          <t>Glen Waverley Line</t>
         </is>
       </c>
       <c r="D1673" t="inlineStr">
@@ -63211,7 +63211,7 @@
       <c r="B1680" t="inlineStr"/>
       <c r="C1680" t="inlineStr">
         <is>
-          <t>Glen Waverley Line</t>
+          <t>Lilydale Line</t>
         </is>
       </c>
       <c r="D1680" t="inlineStr">
@@ -63463,7 +63463,7 @@
       <c r="B1694" t="inlineStr"/>
       <c r="C1694" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1694" t="inlineStr">
@@ -63535,7 +63535,7 @@
       <c r="B1698" t="inlineStr"/>
       <c r="C1698" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Cranbourne Line</t>
         </is>
       </c>
       <c r="D1698" t="inlineStr">
@@ -63607,7 +63607,7 @@
       <c r="B1702" t="inlineStr"/>
       <c r="C1702" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1702" t="inlineStr">
@@ -63715,7 +63715,7 @@
       <c r="B1708" t="inlineStr"/>
       <c r="C1708" t="inlineStr">
         <is>
-          <t>Sunbury Line</t>
+          <t>Pakenham Line</t>
         </is>
       </c>
       <c r="D1708" t="inlineStr">
@@ -63751,7 +63751,7 @@
       <c r="B1710" t="inlineStr"/>
       <c r="C1710" t="inlineStr">
         <is>
-          <t>Pakenham Line</t>
+          <t>Sunbury Line</t>
         </is>
       </c>
       <c r="D1710" t="inlineStr">
@@ -64465,7 +64465,7 @@
       <c r="B1753" t="inlineStr"/>
       <c r="C1753" t="inlineStr">
         <is>
-          <t>Aurizon Shunter</t>
+          <t>Aurizon Nickel Residue</t>
         </is>
       </c>
       <c r="D1753" t="inlineStr">

</xml_diff>

<commit_message>
Update RailOps database files
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -5953,7 +5953,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -6713,7 +6713,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -7621,7 +7621,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
@@ -8725,7 +8725,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
@@ -8869,7 +8869,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
@@ -8917,7 +8917,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -9109,7 +9109,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
@@ -9157,7 +9157,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr">
@@ -9349,7 +9349,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
@@ -9493,7 +9493,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H189" s="2" t="inlineStr">
@@ -9541,7 +9541,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
@@ -9637,7 +9637,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -9685,7 +9685,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -9733,7 +9733,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -9781,7 +9781,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr">
@@ -9877,7 +9877,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -9925,7 +9925,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
@@ -9973,7 +9973,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr">
@@ -10021,7 +10021,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -10117,7 +10117,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -10165,7 +10165,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -10213,7 +10213,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -10357,7 +10357,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -10405,7 +10405,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
@@ -10453,7 +10453,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
@@ -10597,7 +10597,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
@@ -10645,7 +10645,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr">
@@ -10789,7 +10789,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
@@ -10981,7 +10981,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr">
@@ -11269,7 +11269,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
@@ -11317,7 +11317,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr">
@@ -11405,7 +11405,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr">
@@ -11453,7 +11453,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr">
@@ -11501,7 +11501,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr">
@@ -11549,7 +11549,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr">
@@ -11597,7 +11597,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
@@ -11645,7 +11645,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr">
@@ -11741,7 +11741,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
@@ -11789,7 +11789,7 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
@@ -11885,7 +11885,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr">
@@ -11933,7 +11933,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H241" s="2" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr">
@@ -12121,7 +12121,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
@@ -12217,7 +12217,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12265,7 +12265,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
@@ -12361,7 +12361,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
@@ -12453,7 +12453,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr">
@@ -12645,7 +12645,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T18:28:19.918328Z</t>
+          <t>2026-04-29T18:54:54.320678Z</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update RailOps database files - 2026-05-02 14:32:10 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -541,17 +541,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>-32.83151</t>
+          <t>-32.91891</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>151.685187</t>
+          <t>151.740053</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -685,17 +685,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-33.95803</t>
+          <t>-33.920067</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>151.21896</t>
+          <t>151.168067</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>-30.676417</t>
+          <t>-30.71328</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>129.839493</t>
+          <t>129.491933</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2017,17 +2017,17 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T10:33:54.109373Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>-34.216883</t>
+          <t>-34.217833</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>150.592413</t>
+          <t>150.59216</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2353,17 +2353,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>-34.173343</t>
+          <t>-34.180087</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>150.605</t>
+          <t>150.61296</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>-34.212737</t>
+          <t>-34.184703</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>150.595373</t>
+          <t>150.613733</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3021,17 +3021,17 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>-32.903</t>
+          <t>-32.903037</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>151.755093</t>
+          <t>151.755253</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3213,17 +3213,17 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>-30.974423</t>
+          <t>-31.16243</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>150.241933</t>
+          <t>150.316373</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3338,12 +3338,12 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>5524</t>
+          <t>5525</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>5524 North West NSW North West NSW</t>
+          <t>5525 North West NSW North West NSW</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>-31.345873</t>
+          <t>-31.346707</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>150.642173</t>
+          <t>150.634227</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>-31.11855</t>
+          <t>-31.248227</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>150.270933</t>
+          <t>150.46812</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3497,17 +3497,17 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>-32.67131</t>
+          <t>-32.64319</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>151.370667</t>
+          <t>151.227373</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3593,17 +3593,17 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>-32.40719</t>
+          <t>-32.43322</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>151.021627</t>
+          <t>151.0558</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>-32.633097</t>
+          <t>-32.632603</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>151.109467</t>
+          <t>151.110493</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>-32.866493</t>
+          <t>-32.718387</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>151.700387</t>
+          <t>151.467933</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>-32.66424</t>
+          <t>-32.442113</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>151.249653</t>
+          <t>151.05764</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3929,17 +3929,17 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T12:31:56.578266Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>-31.35379</t>
+          <t>-31.677487</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>150.604747</t>
+          <t>150.752307</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3977,17 +3977,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-31.464153</t>
+          <t>-31.64995</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>150.67516</t>
+          <t>150.72604</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4025,17 +4025,17 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>-31.777937</t>
+          <t>-31.874753</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>150.80056</t>
+          <t>150.882867</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4121,12 +4121,12 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>-30.549543</t>
+          <t>-30.549547</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4309,17 +4309,17 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>-30.778072</t>
+          <t>-30.778095</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>121.421761</t>
+          <t>121.421753</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -4405,17 +4405,17 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T08:03:36.971806Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>-31.958173</t>
+          <t>-31.95775</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>141.46956</t>
+          <t>141.480173</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -4549,17 +4549,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>-30.976377</t>
+          <t>-30.937883</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>126.6046</t>
+          <t>127.124933</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4645,17 +4645,17 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>-31.006153</t>
+          <t>-31.00981</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>125.124107</t>
+          <t>124.603307</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4693,17 +4693,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>-37.813917</t>
+          <t>-37.89165</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>144.854853</t>
+          <t>144.68008</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -4789,17 +4789,17 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>-36.64515</t>
+          <t>-36.645153</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>142.28084</t>
+          <t>142.280827</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4837,17 +4837,17 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>-34.099737</t>
+          <t>-33.77061</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>138.237413</t>
+          <t>138.216093</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4885,17 +4885,17 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>-30.887383</t>
+          <t>-30.84112</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>120.907813</t>
+          <t>121.210533</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -5394,12 +5394,12 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>8874</t>
+          <t>8873</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>8874 Western NSW Manildra</t>
+          <t>8873 Manildra Western NSW</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -5409,17 +5409,17 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T10:33:54.109373Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>-33.186723</t>
+          <t>-33.18168</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>148.69404</t>
+          <t>148.67092</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -5457,17 +5457,17 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>-33.965</t>
+          <t>-33.969757</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>151.217027</t>
+          <t>151.221293</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -5601,17 +5601,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>-33.701053</t>
+          <t>-33.710623</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>150.561053</t>
+          <t>150.35684</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>-31.03001</t>
+          <t>-31.02326</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>123.48736</t>
+          <t>123.094493</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -6273,17 +6273,17 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>-36.372497</t>
+          <t>-36.47974</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>141.878907</t>
+          <t>142.059147</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -6369,17 +6369,17 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>-32.134087</t>
+          <t>-31.870467</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>137.448813</t>
+          <t>137.343053</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -6706,17 +6706,17 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>-33.486823</t>
+          <t>-33.47976</t>
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>150.030533</t>
+          <t>150.13716</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -6835,12 +6835,12 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>T171</t>
+          <t>T170</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>T171 Port Botany Enfield</t>
+          <t>T170 Enfield Port Botany</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -6850,17 +6850,17 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01T21:03:03.212633Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>-33.902957</t>
+          <t>-33.90783</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>151.073773</t>
+          <t>151.081133</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -6994,17 +6994,17 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>-33.112607</t>
+          <t>-33.258843</t>
         </is>
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>138.62148</t>
+          <t>138.36008</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -7118,17 +7118,17 @@
       <c r="B140" s="2" t="inlineStr"/>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>PN Light Engine Movement</t>
+          <t>PN Light Engine</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>0506</t>
+          <t>0505</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>0506</t>
+          <t>0505</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -7138,17 +7138,17 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>-37.805767</t>
+          <t>-37.805083</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>144.932667</t>
+          <t>144.939293</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -7378,17 +7378,17 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>-20.573748</t>
+          <t>-21.041703</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>134.18924</t>
+          <t>134.210853</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -7474,17 +7474,17 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>-31.41465</t>
+          <t>-31.239023</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>136.9612</t>
+          <t>136.691947</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -7570,17 +7570,17 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>-34.997283</t>
+          <t>-34.999067</t>
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>138.637213</t>
+          <t>138.602187</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -7666,17 +7666,17 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>-30.081597</t>
+          <t>-30.441803</t>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>134.53548</t>
+          <t>134.52376</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -7714,17 +7714,17 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>-32.401673</t>
+          <t>-32.478977</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>137.74076</t>
+          <t>137.77276</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -7762,17 +7762,17 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>-32.72525</t>
+          <t>-32.657307</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>151.511133</t>
+          <t>151.282093</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -7810,17 +7810,17 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>-32.490403</t>
+          <t>-32.63128</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>151.13692</t>
+          <t>151.227973</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -7858,17 +7858,17 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>-32.273397</t>
+          <t>-32.273347</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>149.762307</t>
+          <t>149.765427</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -7906,17 +7906,17 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>-32.6594</t>
+          <t>-32.494713</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>151.32368</t>
+          <t>151.137173</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>-32.658467</t>
+          <t>-32.72264</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>151.28744</t>
+          <t>151.500373</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -8670,17 +8670,17 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>-32.39136</t>
+          <t>-32.391513</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>151.0016</t>
+          <t>150.998573</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
@@ -8718,17 +8718,17 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>-32.874237</t>
+          <t>-32.871453</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>151.703773</t>
+          <t>151.745333</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -8766,17 +8766,17 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>-32.754953</t>
+          <t>-32.837927</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>151.605973</t>
+          <t>151.68792</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -9242,17 +9242,17 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>-34.850407</t>
+          <t>-34.749353</t>
         </is>
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>150.61172</t>
+          <t>150.810853</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -9290,17 +9290,17 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
-          <t>-34.237143</t>
+          <t>-34.42354</t>
         </is>
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>150.983653</t>
+          <t>150.88896</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -9338,17 +9338,17 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>-33.18865</t>
+          <t>-33.186613</t>
         </is>
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>148.58768</t>
+          <t>148.69196</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
@@ -9718,17 +9718,17 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>-34.859593</t>
+          <t>-34.86812</t>
         </is>
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>138.577133</t>
+          <t>138.57564</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -9958,17 +9958,17 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
-          <t>-32.503163</t>
+          <t>-32.46948</t>
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>137.785373</t>
+          <t>137.76836</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -10160,7 +10160,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>137.767827</t>
+          <t>137.7678</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -10198,17 +10198,17 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>-31.621613</t>
+          <t>-31.491737</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>117.825933</t>
+          <t>118.227853</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
@@ -10246,12 +10246,12 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>-31.95894</t>
+          <t>-31.958937</t>
         </is>
       </c>
       <c r="I205" s="2" t="inlineStr">
@@ -10342,17 +10342,17 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>-33.217907</t>
+          <t>-33.140473</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>148.369107</t>
+          <t>148.147347</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
@@ -10438,17 +10438,17 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>-30.50632</t>
+          <t>-30.51259</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>132.25636</t>
+          <t>132.614413</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -10486,17 +10486,17 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>-30.619407</t>
+          <t>-30.558257</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>133.875307</t>
+          <t>133.543307</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr">
@@ -10534,17 +10534,17 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>-32.91662</t>
+          <t>-32.898793</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>151.743</t>
+          <t>151.760227</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -10582,17 +10582,17 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>-30.855677</t>
+          <t>-30.828967</t>
         </is>
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>120.695893</t>
+          <t>120.259147</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -10630,17 +10630,17 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
-          <t>-28.606893</t>
+          <t>-28.858417</t>
         </is>
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>152.991507</t>
+          <t>153.038707</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -10678,17 +10678,17 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>-30.79242</t>
+          <t>-30.738493</t>
         </is>
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>128.7132</t>
+          <t>129.249413</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -10918,17 +10918,17 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>-32.482387</t>
+          <t>-32.54149</t>
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>137.770947</t>
+          <t>137.8576</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -11062,17 +11062,17 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t>-33.83531</t>
+          <t>-33.886267</t>
         </is>
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>151.016147</t>
+          <t>151.054293</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -11254,17 +11254,17 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>-33.13678</t>
+          <t>-33.13399</t>
         </is>
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>148.098107</t>
+          <t>148.099387</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -11302,17 +11302,17 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
-          <t>-30.995483</t>
+          <t>-31.012587</t>
         </is>
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>126.33076</t>
+          <t>125.808653</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr">
@@ -11350,17 +11350,17 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
-          <t>-30.612827</t>
+          <t>-30.577227</t>
         </is>
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>130.41568</t>
+          <t>130.726373</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr">
@@ -11398,17 +11398,17 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
-          <t>-33.128683</t>
+          <t>-33.137023</t>
         </is>
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>148.106107</t>
+          <t>148.098067</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr">
@@ -11494,17 +11494,17 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t>-36.900863</t>
+          <t>-36.813493</t>
         </is>
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>142.66068</t>
+          <t>142.592307</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr">
@@ -11734,17 +11734,17 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>-34.459167</t>
+          <t>-34.445927</t>
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>150.8766</t>
+          <t>150.88276</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -11782,17 +11782,17 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
-          <t>-34.44897</t>
+          <t>-34.447327</t>
         </is>
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>150.879707</t>
+          <t>150.880173</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -11830,17 +11830,17 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
-          <t>-33.926193</t>
+          <t>-33.874437</t>
         </is>
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>151.181867</t>
+          <t>151.06644</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -11922,17 +11922,17 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
-          <t>-28.953201</t>
+          <t>-28.95269</t>
         </is>
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>121.51709</t>
+          <t>121.517075</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -11970,17 +11970,17 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
-          <t>-30.777304</t>
+          <t>-30.777319</t>
         </is>
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>121.422951</t>
+          <t>121.42292</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -12306,17 +12306,17 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>-32.247317</t>
+          <t>-32.255557</t>
         </is>
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>148.61964</t>
+          <t>148.521627</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -12402,17 +12402,17 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>-32.928173</t>
+          <t>-32.929703</t>
         </is>
       </c>
       <c r="I250" s="2" t="inlineStr">
         <is>
-          <t>151.727093</t>
+          <t>151.72532</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr">
@@ -12531,12 +12531,12 @@
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>C79T</t>
+          <t>C81T</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>C79T brisbane-roma-st townsville</t>
+          <t>C81T brisbane-roma-st cairns</t>
         </is>
       </c>
       <c r="F253" s="2" t="inlineStr">
@@ -12546,17 +12546,17 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T11:33:58.854165Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
-          <t>-24.629022</t>
+          <t>-23.368893</t>
         </is>
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>151.911587</t>
+          <t>150.507735</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -12874,17 +12874,17 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>-33.040297</t>
+          <t>-33.014643</t>
         </is>
       </c>
       <c r="I260" s="2" t="inlineStr">
         <is>
-          <t>146.168667</t>
+          <t>145.677973</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr">
@@ -12970,17 +12970,17 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
-          <t>-31.00939</t>
+          <t>-31.011943</t>
         </is>
       </c>
       <c r="I262" s="2" t="inlineStr">
         <is>
-          <t>125.411533</t>
+          <t>125.70256</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr">
@@ -13402,17 +13402,17 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
-          <t>-32.704017</t>
+          <t>-32.572517</t>
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>151.401987</t>
+          <t>151.16616</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -13546,17 +13546,17 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
-          <t>-31.718007</t>
+          <t>-31.66549</t>
         </is>
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>150.78376</t>
+          <t>150.739373</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -13594,17 +13594,17 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr">
         <is>
-          <t>-32.269007</t>
+          <t>-32.336717</t>
         </is>
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>149.80248</t>
+          <t>149.94624</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -13690,17 +13690,17 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr">
         <is>
-          <t>-32.266447</t>
+          <t>-32.369763</t>
         </is>
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>150.881213</t>
+          <t>151.02092</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -13738,12 +13738,12 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>-32.281313</t>
+          <t>-32.281303</t>
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr">
@@ -13786,17 +13786,17 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t>-32.7846</t>
+          <t>-32.876757</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>151.640947</t>
+          <t>151.7132</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -13834,17 +13834,17 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>-32.446907</t>
+          <t>-32.36889</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>150.17232</t>
+          <t>149.997627</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -14122,17 +14122,17 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>-32.893137</t>
+          <t>-32.732627</t>
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>151.718</t>
+          <t>151.536587</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -14587,12 +14587,12 @@
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>0959</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>8158 Wendouree Southern Cross</t>
+          <t>0959</t>
         </is>
       </c>
       <c r="F296" s="2" t="inlineStr">
@@ -14602,17 +14602,17 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:03:19.673293Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
-          <t>-37.811307</t>
+          <t>-37.799373</t>
         </is>
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>144.94572</t>
+          <t>144.922107</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
@@ -14923,12 +14923,12 @@
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>0958</t>
+          <t>0959</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>0958</t>
+          <t>0959</t>
         </is>
       </c>
       <c r="F303" s="2" t="inlineStr">
@@ -14938,17 +14938,17 @@
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H303" s="2" t="inlineStr">
         <is>
-          <t>-37.80612</t>
+          <t>-37.80426</t>
         </is>
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>144.934907</t>
+          <t>144.93804</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -15158,17 +15158,17 @@
       <c r="B308" s="2" t="inlineStr"/>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Western Line Service</t>
+          <t>Empty Car Transfer for Maintenance</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>8186</t>
+          <t>8198</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>8186 Ararat Southern Cross</t>
+          <t>8198 Ballarat Bombardier Melbourne (Via Geelong)</t>
         </is>
       </c>
       <c r="F308" s="2" t="inlineStr">
@@ -15178,17 +15178,17 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T06:31:11.501259Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>-37.798807</t>
+          <t>-37.808847</t>
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>144.919307</t>
+          <t>144.94356</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -16450,17 +16450,17 @@
       <c r="B335" s="2" t="inlineStr"/>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>Northern Line Service</t>
+          <t>Western Line Service</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>8056</t>
+          <t>8165</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>8056 Bendigo (M-Sa) Southern Cross</t>
+          <t>8165 Southern Cross Sttaion Wendouree Station</t>
         </is>
       </c>
       <c r="F335" s="2" t="inlineStr">
@@ -16470,17 +16470,17 @@
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>-37.812927</t>
+          <t>-37.7998</t>
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>144.947667</t>
+          <t>144.866493</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
@@ -17127,12 +17127,12 @@
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>8807</t>
+          <t>8819</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
         <is>
-          <t>8807 Southern Cross Waurn Ponds</t>
+          <t>8819 Southern Cross Waurn Ponds</t>
         </is>
       </c>
       <c r="F349" s="2" t="inlineStr">
@@ -17142,17 +17142,17 @@
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T11:33:58.854165Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H349" s="2" t="inlineStr">
         <is>
-          <t>-38.068817</t>
+          <t>-37.786563</t>
         </is>
       </c>
       <c r="I349" s="2" t="inlineStr">
         <is>
-          <t>144.382133</t>
+          <t>144.831027</t>
         </is>
       </c>
       <c r="J349" s="2" t="inlineStr">
@@ -17334,17 +17334,17 @@
       </c>
       <c r="G353" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H353" s="2" t="inlineStr">
         <is>
-          <t>-37.786517</t>
+          <t>-37.96292</t>
         </is>
       </c>
       <c r="I353" s="2" t="inlineStr">
         <is>
-          <t>144.830973</t>
+          <t>144.49868</t>
         </is>
       </c>
       <c r="J353" s="2" t="inlineStr">
@@ -17666,17 +17666,17 @@
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H360" s="2" t="inlineStr">
         <is>
-          <t>-30.165693</t>
+          <t>-29.865233</t>
         </is>
       </c>
       <c r="I360" s="2" t="inlineStr">
         <is>
-          <t>153.01308</t>
+          <t>152.999907</t>
         </is>
       </c>
       <c r="J360" s="2" t="inlineStr">
@@ -17714,17 +17714,17 @@
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H361" s="2" t="inlineStr">
         <is>
-          <t>-31.176977</t>
+          <t>-31.467787</t>
         </is>
       </c>
       <c r="I361" s="2" t="inlineStr">
         <is>
-          <t>152.8428</t>
+          <t>152.735773</t>
         </is>
       </c>
       <c r="J361" s="2" t="inlineStr">
@@ -18179,12 +18179,12 @@
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>BC407</t>
+          <t>ER408</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
         <is>
-          <t>BC407 Vales Point / Eraring Bulga</t>
+          <t>ER408 Various Mines Eraring</t>
         </is>
       </c>
       <c r="F371" s="2" t="inlineStr">
@@ -18194,17 +18194,17 @@
       </c>
       <c r="G371" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H371" s="2" t="inlineStr">
         <is>
-          <t>-32.67177</t>
+          <t>-32.648743</t>
         </is>
       </c>
       <c r="I371" s="2" t="inlineStr">
         <is>
-          <t>151.12404</t>
+          <t>151.117987</t>
         </is>
       </c>
       <c r="J371" s="2" t="inlineStr">
@@ -18227,12 +18227,12 @@
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>UL128</t>
+          <t>RV115</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
         <is>
-          <t>UL128 Ulan PWCS Kooragang</t>
+          <t>RV115 PWCS Kooragang Ravensworth</t>
         </is>
       </c>
       <c r="F372" s="2" t="inlineStr">
@@ -18242,17 +18242,17 @@
       </c>
       <c r="G372" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H372" s="2" t="inlineStr">
         <is>
-          <t>-32.86868</t>
+          <t>-32.86646</t>
         </is>
       </c>
       <c r="I372" s="2" t="inlineStr">
         <is>
-          <t>151.757827</t>
+          <t>151.75204</t>
         </is>
       </c>
       <c r="J372" s="2" t="inlineStr">
@@ -18338,17 +18338,17 @@
       </c>
       <c r="G374" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H374" s="2" t="inlineStr">
         <is>
-          <t>-32.71855</t>
+          <t>-32.759463</t>
         </is>
       </c>
       <c r="I374" s="2" t="inlineStr">
         <is>
-          <t>151.41296</t>
+          <t>151.61144</t>
         </is>
       </c>
       <c r="J374" s="2" t="inlineStr">
@@ -18386,17 +18386,17 @@
       </c>
       <c r="G375" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H375" s="2" t="inlineStr">
         <is>
-          <t>-32.657127</t>
+          <t>-32.723657</t>
         </is>
       </c>
       <c r="I375" s="2" t="inlineStr">
         <is>
-          <t>151.2818</t>
+          <t>151.497187</t>
         </is>
       </c>
       <c r="J375" s="2" t="inlineStr">
@@ -18419,12 +18419,12 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>RV284</t>
+          <t>UL109</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
         <is>
-          <t>RV284 Ravensworth PWCS Kooragang</t>
+          <t>UL109 PWCS Kooragang Ulan</t>
         </is>
       </c>
       <c r="F376" s="2" t="inlineStr">
@@ -18434,17 +18434,17 @@
       </c>
       <c r="G376" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T13:32:01.324108Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H376" s="2" t="inlineStr">
         <is>
-          <t>-32.86773</t>
+          <t>-32.878827</t>
         </is>
       </c>
       <c r="I376" s="2" t="inlineStr">
         <is>
-          <t>151.753467</t>
+          <t>151.7098</t>
         </is>
       </c>
       <c r="J376" s="2" t="inlineStr">
@@ -18482,17 +18482,17 @@
       </c>
       <c r="G377" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H377" s="2" t="inlineStr">
         <is>
-          <t>-32.324777</t>
+          <t>-32.3367</t>
         </is>
       </c>
       <c r="I377" s="2" t="inlineStr">
         <is>
-          <t>150.713373</t>
+          <t>150.72248</t>
         </is>
       </c>
       <c r="J377" s="2" t="inlineStr">
@@ -18530,17 +18530,17 @@
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:03:07.145457Z</t>
+          <t>2026-05-02T14:32:09.626974Z</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
         <is>
-          <t>-32.394427</t>
+          <t>-32.32073</t>
         </is>
       </c>
       <c r="I378" s="2" t="inlineStr">
         <is>
-          <t>150.677093</t>
+          <t>150.7456</t>
         </is>
       </c>
       <c r="J378" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update RailOps database files - 2026-05-02 16:34:09 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -589,17 +589,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-34.472627</t>
+          <t>-34.341573</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>150.88656</t>
+          <t>150.915027</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-34.303467</t>
+          <t>-34.2988</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>150.590213</t>
+          <t>150.58708</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -821,17 +821,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-34.304727</t>
+          <t>-34.299093</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>150.591547</t>
+          <t>150.58736</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1445,17 +1445,17 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>-32.824987</t>
+          <t>-32.82497</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>151.681173</t>
+          <t>151.681187</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>-30.76787</t>
+          <t>-30.79245</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>128.961</t>
+          <t>128.71324</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:32:09.626974Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>-34.217833</t>
+          <t>-34.22111</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>150.59216</t>
+          <t>150.591173</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2257,17 +2257,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>-33.941183</t>
+          <t>-33.918857</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>150.917347</t>
+          <t>150.933947</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2497,17 +2497,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>-33.949653</t>
+          <t>-33.92214</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>150.91208</t>
+          <t>150.930667</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3069,17 +3069,17 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>-32.90316</t>
+          <t>-32.903073</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>151.755173</t>
+          <t>151.755107</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -3261,17 +3261,17 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>-31.189637</t>
+          <t>-31.189653</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>150.351387</t>
+          <t>150.351373</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>-31.348467</t>
+          <t>-31.224233</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>150.620267</t>
+          <t>150.4112</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3449,17 +3449,17 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>-31.674227</t>
+          <t>-31.674233</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>150.747413</t>
+          <t>150.7474</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3545,17 +3545,17 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>-32.046563</t>
+          <t>-31.835277</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>150.866933</t>
+          <t>150.921387</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>-32.722163</t>
+          <t>-32.775257</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>151.417413</t>
+          <t>151.62996</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>-32.630317</t>
+          <t>-32.662253</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>151.227747</t>
+          <t>151.345747</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>-30.971273</t>
+          <t>-31.009097</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>150.239573</t>
+          <t>150.275</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:32:09.626974Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>-32.718387</t>
+          <t>-32.671157</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>151.467933</t>
+          <t>151.37044</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3833,17 +3833,17 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>-31.95819</t>
+          <t>-31.745847</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>150.869</t>
+          <t>150.798533</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>-32.867113</t>
+          <t>-32.83842</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>151.753987</t>
+          <t>151.687547</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3977,17 +3977,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-31.983113</t>
+          <t>-32.073433</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>150.86792</t>
+          <t>150.870013</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4025,17 +4025,17 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>-31.75107</t>
+          <t>-31.772127</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>150.800533</t>
+          <t>150.853933</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4073,17 +4073,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>-32.2813</t>
+          <t>-32.388507</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>150.947573</t>
+          <t>151.029813</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4121,17 +4121,17 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>-32.534737</t>
+          <t>-32.664793</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>151.154573</t>
+          <t>151.311413</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -4169,17 +4169,17 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>-30.612703</t>
+          <t>-30.612817</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>130.416253</t>
+          <t>130.415187</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4357,12 +4357,12 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>-30.778061</t>
+          <t>-30.778076</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4453,17 +4453,17 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>-32.389</t>
+          <t>-32.505867</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>142.441653</t>
+          <t>142.69932</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4549,17 +4549,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>-32.633457</t>
+          <t>-32.861467</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>139.486147</t>
+          <t>139.230453</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4597,17 +4597,17 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T15:34:12.020596Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>-30.831397</t>
+          <t>-30.721253</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>128.310333</t>
+          <t>129.416067</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -4693,17 +4693,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>-31.02351</t>
+          <t>-30.977237</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>123.08408</t>
+          <t>122.648467</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -4741,17 +4741,17 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>-37.99525</t>
+          <t>-37.767643</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>143.5296</t>
+          <t>143.021227</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -4837,12 +4837,12 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>-36.645167</t>
+          <t>-36.645177</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -4933,17 +4933,17 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>-30.740287</t>
+          <t>-30.8477</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>121.515907</t>
+          <t>121.657493</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -5105,17 +5105,17 @@
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Aurizon Loaded Grain</t>
+          <t>Aurizon Wagon Transfer</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>2182S</t>
+          <t>1122S</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>2182S Tailem Bend Viterra, Pelican Point</t>
+          <t>1122S Pelican Point/Port Flat Dry Creek North</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -5125,17 +5125,17 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>-34.77773</t>
+          <t>-34.817497</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>138.504293</t>
+          <t>138.507693</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5313,17 +5313,17 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>-33.888413</t>
+          <t>-33.894337</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>151.201613</t>
+          <t>151.19356</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -5457,17 +5457,17 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>-32.946223</t>
+          <t>-32.65973</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>148.164947</t>
+          <t>148.168747</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -5505,17 +5505,17 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>-33.959213</t>
+          <t>-33.963463</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>151.21888</t>
+          <t>151.219707</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -5649,17 +5649,17 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>-33.250383</t>
+          <t>-33.107103</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>150.016973</t>
+          <t>149.99264</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -5697,17 +5697,17 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>-34.47268</t>
+          <t>-34.347187</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>150.886973</t>
+          <t>150.916133</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -5937,17 +5937,17 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>-30.920173</t>
+          <t>-30.858623</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>122.092093</t>
+          <t>121.682773</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -5985,17 +5985,17 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>-32.372097</t>
+          <t>-32.50087</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>137.633187</t>
+          <t>137.834587</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -6081,17 +6081,17 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>-30.307453</t>
+          <t>-30.307527</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>149.777093</t>
+          <t>149.77704</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -6369,17 +6369,17 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>-36.70748</t>
+          <t>-36.634663</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>142.201413</t>
+          <t>142.483933</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -6417,17 +6417,17 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>-31.575943</t>
+          <t>-31.640633</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>116.350613</t>
+          <t>116.597653</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -6465,17 +6465,17 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>-31.48184</t>
+          <t>-31.422307</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>137.058507</t>
+          <t>136.99352</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -6802,17 +6802,17 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>-33.719917</t>
+          <t>-33.702113</t>
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>150.447227</t>
+          <t>150.573627</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -7090,17 +7090,17 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>-33.916617</t>
+          <t>-34.17401</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>138.229867</t>
+          <t>138.274987</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -7474,17 +7474,17 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>-22.299795</t>
+          <t>-22.780063</t>
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>133.911147</t>
+          <t>133.819773</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -7522,17 +7522,17 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>-24.644872</t>
+          <t>-24.321218</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>133.708893</t>
+          <t>133.728</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -7570,17 +7570,17 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>-30.963547</t>
+          <t>-30.907427</t>
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>135.479067</t>
+          <t>135.299587</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -7714,17 +7714,17 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>-12.49814</t>
+          <t>-12.8441</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>130.955253</t>
+          <t>131.134947</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -7762,17 +7762,17 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>-30.858717</t>
+          <t>-30.938877</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>135.028653</t>
+          <t>135.408027</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -7810,17 +7810,17 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>-32.838997</t>
+          <t>-32.94231</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>137.98244</t>
+          <t>137.982867</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -7858,17 +7858,17 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>-32.33414</t>
+          <t>-32.334757</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>150.89904</t>
+          <t>150.900173</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
@@ -7939,12 +7939,12 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>UL303</t>
+          <t>UL304</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>UL303 PWCS Kooragang Ulan</t>
+          <t>UL304 Ulan PWCS Kooragang</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>-32.270633</t>
+          <t>-32.32381</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>149.774427</t>
+          <t>149.92744</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -8002,17 +8002,17 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>-32.407243</t>
+          <t>-32.410023</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>151.095013</t>
+          <t>151.094053</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -8050,17 +8050,17 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T15:34:12.020596Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>-32.867137</t>
+          <t>-32.8749</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>151.756627</t>
+          <t>151.772867</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -8098,17 +8098,17 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>-32.49627</t>
+          <t>-32.697463</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>137.692987</t>
+          <t>137.515773</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -8558,17 +8558,17 @@
       <c r="B170" s="2" t="inlineStr"/>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Empty Car Transfer</t>
+          <t>Hunter Line Service</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>V874</t>
+          <t>V703</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>V874 Newcastle Interchange Broadmeadow Maintenance Centre</t>
+          <t>V703 Newcastle Interchange Telarah</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -8578,17 +8578,17 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T11:33:58.854165Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>-32.928377</t>
+          <t>-32.90366</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>151.72536</t>
+          <t>151.7326</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -8814,17 +8814,17 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>-32.48299</t>
+          <t>-32.630437</t>
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>151.134667</t>
+          <t>151.227867</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -8862,17 +8862,17 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>-32.87436</t>
+          <t>-32.739973</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>151.703773</t>
+          <t>151.58172</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -8910,17 +8910,17 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>-32.87077</t>
+          <t>-32.868013</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>151.760613</t>
+          <t>151.754027</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -9098,17 +9098,17 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>-31.569243</t>
+          <t>-31.67682</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>116.410493</t>
+          <t>116.136213</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -9386,17 +9386,17 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>-34.480093</t>
+          <t>-34.27788</t>
         </is>
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>150.80384</t>
+          <t>150.951187</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr">
@@ -9622,17 +9622,17 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>-33.88618</t>
+          <t>-33.893013</t>
         </is>
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>151.203707</t>
+          <t>151.196987</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
@@ -10150,17 +10150,17 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>-32.225593</t>
+          <t>-31.884333</t>
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>137.53428</t>
+          <t>137.350907</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
@@ -10342,12 +10342,12 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>-32.469087</t>
+          <t>-32.46908</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
@@ -10390,17 +10390,17 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>-31.353143</t>
+          <t>-31.272587</t>
         </is>
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>119.019707</t>
+          <t>119.151547</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
@@ -10438,17 +10438,17 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>-31.957313</t>
+          <t>-32.14603</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>141.768933</t>
+          <t>142.123573</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
@@ -10534,17 +10534,17 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>-33.135643</t>
+          <t>-33.13562</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>148.135093</t>
+          <t>148.135107</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -10630,17 +10630,17 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
-          <t>-30.542187</t>
+          <t>-30.571357</t>
         </is>
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>133.281173</t>
+          <t>133.5992</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
@@ -10678,17 +10678,17 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>-30.494333</t>
+          <t>-30.49179</t>
         </is>
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>132.49012</t>
+          <t>132.33372</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -10726,17 +10726,17 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
-          <t>-32.898873</t>
+          <t>-32.898837</t>
         </is>
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>151.761627</t>
+          <t>151.7616</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -10774,17 +10774,17 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>-31.273733</t>
+          <t>-31.35359</t>
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>119.146213</t>
+          <t>118.989707</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -10822,17 +10822,17 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>-29.5853</t>
+          <t>-29.67604</t>
         </is>
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>152.969093</t>
+          <t>152.919613</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -10870,12 +10870,12 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>-30.612837</t>
+          <t>-30.61283</t>
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr">
@@ -11110,17 +11110,17 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t>-33.339313</t>
+          <t>-33.183883</t>
         </is>
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>138.25656</t>
+          <t>138.50472</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -11446,12 +11446,12 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
-          <t>-33.13399</t>
+          <t>-33.134007</t>
         </is>
       </c>
       <c r="I230" s="2" t="inlineStr">
@@ -11494,7 +11494,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr">
@@ -11542,17 +11542,17 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
-          <t>-31.03375</t>
+          <t>-31.032983</t>
         </is>
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>124.122027</t>
+          <t>123.624947</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr">
@@ -11590,17 +11590,17 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
-          <t>-30.492303</t>
+          <t>-30.48599</t>
         </is>
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>132.139987</t>
+          <t>132.41852</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr">
@@ -11638,17 +11638,17 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>-33.139617</t>
+          <t>-33.111377</t>
         </is>
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>148.097493</t>
+          <t>147.847987</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -11734,17 +11734,17 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>-36.42103</t>
+          <t>-36.35993</t>
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>142.002893</t>
+          <t>141.78696</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -11974,17 +11974,17 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H241" s="2" t="inlineStr">
         <is>
-          <t>-34.4562</t>
+          <t>-34.455493</t>
         </is>
       </c>
       <c r="I241" s="2" t="inlineStr">
         <is>
-          <t>150.875893</t>
+          <t>150.875373</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -12022,17 +12022,17 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>-34.459163</t>
+          <t>-34.463443</t>
         </is>
       </c>
       <c r="I242" s="2" t="inlineStr">
         <is>
-          <t>150.87728</t>
+          <t>150.87508</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr">
@@ -12070,17 +12070,17 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
-          <t>-33.443327</t>
+          <t>-33.150447</t>
         </is>
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>151.329307</t>
+          <t>151.486973</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr">
@@ -12162,17 +12162,17 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
-          <t>-28.938202</t>
+          <t>-28.93948</t>
         </is>
       </c>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>121.516838</t>
+          <t>121.516724</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -12210,17 +12210,17 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
-          <t>-30.777351</t>
+          <t>-30.777369</t>
         </is>
       </c>
       <c r="I246" s="2" t="inlineStr">
         <is>
-          <t>121.422913</t>
+          <t>121.422897</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr">
@@ -12546,17 +12546,17 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
-          <t>-31.841397</t>
+          <t>-31.668587</t>
         </is>
       </c>
       <c r="I253" s="2" t="inlineStr">
         <is>
-          <t>147.723</t>
+          <t>147.396227</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr">
@@ -13018,17 +13018,17 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T02:03:43.962023Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
-          <t>-32.237353</t>
+          <t>-33.18671</t>
         </is>
       </c>
       <c r="I263" s="2" t="inlineStr">
         <is>
-          <t>148.247853</t>
+          <t>148.69308</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr">
@@ -13114,17 +13114,17 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>-32.9535</t>
+          <t>-32.887877</t>
         </is>
       </c>
       <c r="I265" s="2" t="inlineStr">
         <is>
-          <t>144.57568</t>
+          <t>144.019933</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr">
@@ -13210,17 +13210,17 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>-30.94269</t>
+          <t>-30.893127</t>
         </is>
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>127.068533</t>
+          <t>127.63972</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -13258,17 +13258,17 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>-23.651903</t>
+          <t>-23.724971</t>
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>150.0987</t>
+          <t>149.844241</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -13642,17 +13642,17 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
         <is>
-          <t>-32.394153</t>
+          <t>-32.39225</t>
         </is>
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>151.00588</t>
+          <t>151.003227</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -13786,17 +13786,17 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t>-31.738447</t>
+          <t>-31.669457</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>150.78856</t>
+          <t>150.741893</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -13834,17 +13834,17 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>-32.423127</t>
+          <t>-32.361253</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>150.275347</t>
+          <t>150.495893</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -13930,17 +13930,17 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
         <is>
-          <t>-32.663583</t>
+          <t>-32.73935</t>
         </is>
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>151.350027</t>
+          <t>151.555453</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
@@ -13978,17 +13978,17 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t>-32.28732</t>
+          <t>-32.28678</t>
         </is>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>150.8232</t>
+          <t>150.826547</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -14026,17 +14026,17 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
-          <t>-32.86871</t>
+          <t>-32.86737</t>
         </is>
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>151.758027</t>
+          <t>151.755</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -14074,17 +14074,17 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>-32.26349</t>
+          <t>-32.264867</t>
         </is>
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>149.79184</t>
+          <t>149.795227</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -14122,17 +14122,17 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>-32.658327</t>
+          <t>-32.433777</t>
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>151.236653</t>
+          <t>151.055853</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -14170,17 +14170,17 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
-          <t>-30.564287</t>
+          <t>-30.56723</t>
         </is>
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>150.117613</t>
+          <t>150.116093</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -14218,17 +14218,17 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>-32.392167</t>
+          <t>-32.49559</t>
         </is>
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>151.03124</t>
+          <t>151.137107</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -14362,17 +14362,17 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>-32.634903</t>
+          <t>-32.633293</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>151.105747</t>
+          <t>151.109093</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -14794,17 +14794,17 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>-37.798797</t>
+          <t>-37.815123</t>
         </is>
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>144.9192</t>
+          <t>144.94988</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -15610,17 +15610,17 @@
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H317" s="2" t="inlineStr">
         <is>
-          <t>-38.020527</t>
+          <t>-38.10632</t>
         </is>
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>144.416093</t>
+          <t>144.357947</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
@@ -16662,17 +16662,17 @@
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H339" s="2" t="inlineStr">
         <is>
-          <t>-37.79878</t>
+          <t>-37.816047</t>
         </is>
       </c>
       <c r="I339" s="2" t="inlineStr">
         <is>
-          <t>144.919107</t>
+          <t>144.950733</t>
         </is>
       </c>
       <c r="J339" s="2" t="inlineStr">
@@ -17906,17 +17906,17 @@
       </c>
       <c r="G365" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H365" s="2" t="inlineStr">
         <is>
-          <t>-29.046593</t>
+          <t>-28.723207</t>
         </is>
       </c>
       <c r="I365" s="2" t="inlineStr">
         <is>
-          <t>152.960813</t>
+          <t>152.996067</t>
         </is>
       </c>
       <c r="J365" s="2" t="inlineStr">
@@ -17954,17 +17954,17 @@
       </c>
       <c r="G366" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H366" s="2" t="inlineStr">
         <is>
-          <t>-31.908543</t>
+          <t>-32.00383</t>
         </is>
       </c>
       <c r="I366" s="2" t="inlineStr">
         <is>
-          <t>152.2124</t>
+          <t>151.96736</t>
         </is>
       </c>
       <c r="J366" s="2" t="inlineStr">
@@ -18434,17 +18434,17 @@
       </c>
       <c r="G376" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H376" s="2" t="inlineStr">
         <is>
-          <t>-32.835873</t>
+          <t>-32.94297</t>
         </is>
       </c>
       <c r="I376" s="2" t="inlineStr">
         <is>
-          <t>151.687027</t>
+          <t>151.685267</t>
         </is>
       </c>
       <c r="J376" s="2" t="inlineStr">
@@ -18482,17 +18482,17 @@
       </c>
       <c r="G377" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H377" s="2" t="inlineStr">
         <is>
-          <t>-32.509267</t>
+          <t>-32.406053</t>
         </is>
       </c>
       <c r="I377" s="2" t="inlineStr">
         <is>
-          <t>151.152533</t>
+          <t>151.01424</t>
         </is>
       </c>
       <c r="J377" s="2" t="inlineStr">
@@ -18515,12 +18515,12 @@
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>BW268</t>
+          <t>BW961</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
         <is>
-          <t>BW268</t>
+          <t>BW961</t>
         </is>
       </c>
       <c r="F378" s="2" t="inlineStr">
@@ -18530,17 +18530,17 @@
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T15:03:30.203260Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
         <is>
-          <t>-32.86845</t>
+          <t>-32.863313</t>
         </is>
       </c>
       <c r="I378" s="2" t="inlineStr">
         <is>
-          <t>151.75676</t>
+          <t>151.730627</t>
         </is>
       </c>
       <c r="J378" s="2" t="inlineStr">
@@ -18578,17 +18578,17 @@
       </c>
       <c r="G379" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H379" s="2" t="inlineStr">
         <is>
-          <t>-32.871957</t>
+          <t>-32.86968</t>
         </is>
       </c>
       <c r="I379" s="2" t="inlineStr">
         <is>
-          <t>151.76372</t>
+          <t>151.7582</t>
         </is>
       </c>
       <c r="J379" s="2" t="inlineStr">
@@ -18626,17 +18626,17 @@
       </c>
       <c r="G380" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H380" s="2" t="inlineStr">
         <is>
-          <t>-32.868447</t>
+          <t>-32.874977</t>
         </is>
       </c>
       <c r="I380" s="2" t="inlineStr">
         <is>
-          <t>151.761973</t>
+          <t>151.772787</t>
         </is>
       </c>
       <c r="J380" s="2" t="inlineStr">
@@ -18674,17 +18674,17 @@
       </c>
       <c r="G381" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H381" s="2" t="inlineStr">
         <is>
-          <t>-32.303043</t>
+          <t>-32.37869</t>
         </is>
       </c>
       <c r="I381" s="2" t="inlineStr">
         <is>
-          <t>150.984173</t>
+          <t>150.68692</t>
         </is>
       </c>
       <c r="J381" s="2" t="inlineStr">
@@ -18722,17 +18722,17 @@
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H382" s="2" t="inlineStr">
         <is>
-          <t>-32.342833</t>
+          <t>-32.439303</t>
         </is>
       </c>
       <c r="I382" s="2" t="inlineStr">
         <is>
-          <t>150.98616</t>
+          <t>151.056867</t>
         </is>
       </c>
       <c r="J382" s="2" t="inlineStr">
@@ -18770,17 +18770,17 @@
       </c>
       <c r="G383" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T16:03:27.926022Z</t>
+          <t>2026-05-02T16:34:09.434227Z</t>
         </is>
       </c>
       <c r="H383" s="2" t="inlineStr">
         <is>
-          <t>-32.436583</t>
+          <t>-32.577687</t>
         </is>
       </c>
       <c r="I383" s="2" t="inlineStr">
         <is>
-          <t>151.056387</t>
+          <t>151.17288</t>
         </is>
       </c>
       <c r="J383" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update RailOps database files - 2026-05-02 18:33:10 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -589,17 +589,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-33.920803</t>
+          <t>-33.862047</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>151.157587</t>
+          <t>151.06028</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>T263</t>
+          <t>T260</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>T263 Cooks River Moorebank IMEX Terminal</t>
+          <t>T260 Moorebank IMEX Terminal Port Botany</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -685,17 +685,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T14:32:09.626974Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-33.920067</t>
+          <t>-33.920863</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>151.168067</t>
+          <t>151.170053</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T17:02:28.169445Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-34.3047</t>
+          <t>-34.30507</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>150.591467</t>
+          <t>150.59224</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1445,12 +1445,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>-32.82497</t>
+          <t>-32.82501</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>-30.923627</t>
+          <t>-30.97058</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>127.2914</t>
+          <t>126.733533</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2449,17 +2449,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>-34.213077</t>
+          <t>-34.181967</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>150.59484</t>
+          <t>150.6134</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2497,17 +2497,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>-34.211483</t>
+          <t>-34.18534</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>150.597573</t>
+          <t>150.61384</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3165,17 +3165,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>-32.903063</t>
+          <t>-32.90294</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>151.755107</t>
+          <t>151.755013</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3357,17 +3357,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>-31.189653</t>
+          <t>-31.244587</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>150.351373</t>
+          <t>150.46108</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3497,17 +3497,17 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>-30.96872</t>
+          <t>-30.968647</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>150.23456</t>
+          <t>150.235267</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3545,17 +3545,17 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>-31.988723</t>
+          <t>-32.23993</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>150.867893</t>
+          <t>150.903893</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>-31.675193</t>
+          <t>-31.387727</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>150.748547</t>
+          <t>150.64468</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>-32.873007</t>
+          <t>-32.869847</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>151.76728</t>
+          <t>151.760187</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>-32.872417</t>
+          <t>-32.874593</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>151.734013</t>
+          <t>151.746773</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3833,17 +3833,17 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>-31.35888</t>
+          <t>-31.469543</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>150.645347</t>
+          <t>150.678853</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3929,17 +3929,17 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>-31.34899</t>
+          <t>-31.24373</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>150.64604</t>
+          <t>150.452827</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -4073,17 +4073,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>-32.32978</t>
+          <t>-32.459297</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>150.985</t>
+          <t>151.07904</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4121,17 +4121,17 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>-32.262083</t>
+          <t>-32.34678</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>150.887707</t>
+          <t>150.988107</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -4169,17 +4169,17 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>-32.66044</t>
+          <t>-32.719103</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>151.339653</t>
+          <t>151.485773</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4217,17 +4217,17 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>-32.851907</t>
+          <t>-32.86741</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>151.693933</t>
+          <t>151.75752</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -4265,17 +4265,17 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>-30.67452</t>
+          <t>-30.725373</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>129.85692</t>
+          <t>129.376173</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4453,17 +4453,17 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>-30.778067</t>
+          <t>-30.778051</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>121.421791</t>
+          <t>121.421776</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4549,17 +4549,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>-32.625583</t>
+          <t>-32.80653</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>143.043787</t>
+          <t>143.474133</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4645,17 +4645,17 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>-33.100353</t>
+          <t>-33.278827</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>138.626053</t>
+          <t>138.350867</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4693,17 +4693,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>-30.65038</t>
+          <t>-30.610533</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>130.078813</t>
+          <t>130.435413</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -4789,17 +4789,17 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>-30.85386</t>
+          <t>-30.726487</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>121.671307</t>
+          <t>121.497813</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4837,17 +4837,17 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>-37.11529</t>
+          <t>-37.11317</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>142.805387</t>
+          <t>142.805067</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4933,17 +4933,17 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>-36.64517</t>
+          <t>-36.645163</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>142.28084</t>
+          <t>142.280853</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -4981,17 +4981,17 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>-32.47581</t>
+          <t>-32.469417</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>137.77192</t>
+          <t>137.768333</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -5029,17 +5029,17 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>-30.936953</t>
+          <t>-30.9744</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>122.21852</t>
+          <t>122.575173</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5201,17 +5201,17 @@
       <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Aurizon Wagon Transfer</t>
+          <t>Aurizon Empty Grain</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>1122S</t>
+          <t>1513</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>1122S Pelican Point/Port Flat Dry Creek North</t>
+          <t>1513 Dry Creek North Gladstone</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -5221,17 +5221,17 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>-34.810073</t>
+          <t>-34.809973</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>138.605907</t>
+          <t>138.605987</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -5505,17 +5505,17 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>-36.740283</t>
+          <t>-36.759147</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>142.547867</t>
+          <t>142.559347</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -5601,17 +5601,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>-32.257393</t>
+          <t>-32.244377</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>148.387093</t>
+          <t>148.603387</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5793,17 +5793,17 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>-33.10337</t>
+          <t>-33.103333</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>150.002387</t>
+          <t>149.999973</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>-33.91994</t>
+          <t>-33.862003</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>151.15788</t>
+          <t>151.06012</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -6081,17 +6081,17 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>-30.78284</t>
+          <t>-30.841467</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>121.41264</t>
+          <t>121.167787</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -6129,17 +6129,17 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>-33.16919</t>
+          <t>-33.340803</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>138.05656</t>
+          <t>138.194747</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -6225,17 +6225,17 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>-30.294613</t>
+          <t>-30.377793</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>149.795587</t>
+          <t>149.788507</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6513,17 +6513,17 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>-36.905317</t>
+          <t>-36.945037</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>142.664627</t>
+          <t>142.686827</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -6561,17 +6561,17 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>-31.641877</t>
+          <t>-31.645347</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>117.489733</t>
+          <t>117.623813</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -6609,17 +6609,17 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>-31.366533</t>
+          <t>-31.22809</t>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>136.931067</t>
+          <t>136.663773</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -6946,17 +6946,17 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>-33.8859</t>
+          <t>-33.903683</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>151.068733</t>
+          <t>151.074027</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -7138,17 +7138,17 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>-36.62294</t>
+          <t>-36.624867</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>142.477053</t>
+          <t>142.477787</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -7666,17 +7666,17 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>-23.697963</t>
+          <t>-23.693585</t>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>133.875067</t>
+          <t>133.867733</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -7714,17 +7714,17 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>-30.515247</t>
+          <t>-30.198733</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>134.521587</t>
+          <t>134.53416</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -7810,17 +7810,17 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T17:33:30.507033Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>-34.773247</t>
+          <t>-34.777153</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>138.502893</t>
+          <t>138.504293</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -7858,17 +7858,17 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>-13.570633</t>
+          <t>-13.94227</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>131.721027</t>
+          <t>131.898653</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -7906,17 +7906,17 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>-31.22845</t>
+          <t>-31.220147</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>136.362787</t>
+          <t>136.4446</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>-33.671823</t>
+          <t>-34.008527</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>138.223067</t>
+          <t>138.225947</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -8002,17 +8002,17 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>-32.500553</t>
+          <t>-32.657123</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>151.138627</t>
+          <t>151.28184</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -8050,17 +8050,17 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>-32.874833</t>
+          <t>-32.872297</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>151.7708</t>
+          <t>151.764387</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -8098,17 +8098,17 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>-32.42244</t>
+          <t>-32.414643</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>150.30604</t>
+          <t>150.330907</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -8146,17 +8146,17 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>-32.450117</t>
+          <t>-32.557323</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>151.103253</t>
+          <t>151.157133</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -8434,17 +8434,17 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>-32.87228</t>
+          <t>-32.923523</t>
         </is>
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>151.702827</t>
+          <t>151.757947</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr">
@@ -8578,17 +8578,17 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>-32.9031</t>
+          <t>-32.74145</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>151.732013</t>
+          <t>151.56528</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -8958,17 +8958,17 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>-32.779027</t>
+          <t>-32.870657</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>151.634387</t>
+          <t>151.729427</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -9006,17 +9006,17 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>-32.39875</t>
+          <t>-32.391487</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>151.012187</t>
+          <t>150.998573</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -9054,17 +9054,17 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>-32.735157</t>
+          <t>-32.67177</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>151.54448</t>
+          <t>151.3718</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -9082,17 +9082,17 @@
       <c r="B181" s="2" t="inlineStr"/>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Bathurst Bullet</t>
+          <t>Bathurst Bullet - Transfer</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>WN17</t>
+          <t>WN11</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>WN17 Central Bathurst</t>
+          <t>WN11 Lithgow Bathurst</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
@@ -9102,17 +9102,17 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T12:03:54.495244Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>-33.506413</t>
+          <t>-33.48042</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>149.7492</t>
+          <t>150.158013</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -9178,17 +9178,17 @@
       <c r="B183" s="2" t="inlineStr"/>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Bathurst Bullet</t>
+          <t>Bathurst Bullet - Transfer</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>WN15</t>
+          <t>WN13</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>WN15 Central Bathurst</t>
+          <t>WN13 Lithgow Bathurst</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
@@ -9198,17 +9198,17 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T09:31:09.208054Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>-33.42553</t>
+          <t>-33.476407</t>
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>149.583333</t>
+          <t>150.171307</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -9530,12 +9530,12 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>-33.89074</t>
+          <t>-33.890737</t>
         </is>
       </c>
       <c r="I190" s="2" t="inlineStr">
@@ -10054,17 +10054,17 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>-35.050477</t>
+          <t>-35.112223</t>
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>138.932507</t>
+          <t>139.175027</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -10294,17 +10294,17 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>-31.219223</t>
+          <t>-31.190213</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>136.632533</t>
+          <t>136.27112</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -10486,12 +10486,12 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>-32.46907</t>
+          <t>-32.469067</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
@@ -10534,17 +10534,17 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>-30.828447</t>
+          <t>-30.857247</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>120.249387</t>
+          <t>120.737773</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -10582,17 +10582,17 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>-32.364907</t>
+          <t>-32.44103</t>
         </is>
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>142.410427</t>
+          <t>142.568187</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -10678,17 +10678,17 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>-33.14175</t>
+          <t>-33.129813</t>
         </is>
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>147.95644</t>
+          <t>147.576867</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -10774,17 +10774,17 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>-30.756497</t>
+          <t>-30.876223</t>
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>134.74276</t>
+          <t>135.123427</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -10822,17 +10822,17 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>-30.521023</t>
+          <t>-30.577413</t>
         </is>
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>131.202667</t>
+          <t>130.724387</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -10870,17 +10870,17 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>-32.898837</t>
+          <t>-32.90254</t>
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>151.761627</t>
+          <t>151.76576</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -10918,17 +10918,17 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>-31.408737</t>
+          <t>-31.488177</t>
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>118.415507</t>
+          <t>118.243373</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -10966,17 +10966,17 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>-30.285947</t>
+          <t>-30.473473</t>
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>153.06448</t>
+          <t>153.00952</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -11014,12 +11014,12 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t>-30.61283</t>
+          <t>-30.612827</t>
         </is>
       </c>
       <c r="I221" s="2" t="inlineStr">
@@ -11254,17 +11254,17 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>-32.846633</t>
+          <t>-32.548087</t>
         </is>
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>139.242707</t>
+          <t>139.64668</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -11590,12 +11590,12 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
-          <t>-33.133993</t>
+          <t>-33.133977</t>
         </is>
       </c>
       <c r="I233" s="2" t="inlineStr">
@@ -11638,17 +11638,17 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>-33.55954</t>
+          <t>-33.408903</t>
         </is>
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>151.196893</t>
+          <t>151.348013</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -11686,17 +11686,17 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>-30.97305</t>
+          <t>-30.941337</t>
         </is>
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>122.36852</t>
+          <t>122.241907</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -11734,17 +11734,17 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>-30.55191</t>
+          <t>-30.609</t>
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>133.480373</t>
+          <t>133.832507</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -11782,17 +11782,17 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
-          <t>-33.038927</t>
+          <t>-33.017177</t>
         </is>
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>146.489533</t>
+          <t>146.060373</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -11878,17 +11878,17 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
-          <t>-36.170693</t>
+          <t>-35.896153</t>
         </is>
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>140.47844</t>
+          <t>140.07144</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -12118,17 +12118,17 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>-34.449067</t>
+          <t>-34.44641</t>
         </is>
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>150.88136</t>
+          <t>150.880147</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -12306,17 +12306,17 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>-28.941969</t>
+          <t>-28.942028</t>
         </is>
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>121.516815</t>
+          <t>121.516823</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -12354,17 +12354,17 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
-          <t>-30.777359</t>
+          <t>-30.777313</t>
         </is>
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>121.422897</t>
+          <t>121.422943</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -12690,17 +12690,17 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
-          <t>-31.552923</t>
+          <t>-31.542577</t>
         </is>
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>146.65304</t>
+          <t>146.413187</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -13162,17 +13162,17 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>-33.186653</t>
+          <t>-33.186827</t>
         </is>
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>148.696027</t>
+          <t>148.695707</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -13258,17 +13258,17 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>-32.614417</t>
+          <t>-32.614397</t>
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>143.011427</t>
+          <t>143.011387</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -13354,17 +13354,17 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
-          <t>-30.789367</t>
+          <t>-30.766003</t>
         </is>
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>128.744453</t>
+          <t>128.97948</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -13402,17 +13402,17 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
-          <t>-23.584968</t>
+          <t>-23.593828</t>
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>148.984137</t>
+          <t>148.733895</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -13786,17 +13786,17 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t>-32.391377</t>
+          <t>-32.405407</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>150.996213</t>
+          <t>151.020133</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -13834,17 +13834,17 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>-32.506567</t>
+          <t>-32.29668</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>151.15028</t>
+          <t>150.979027</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -13978,17 +13978,17 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t>-32.281403</t>
+          <t>-32.38384</t>
         </is>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>150.944227</t>
+          <t>151.027947</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -14107,12 +14107,12 @@
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>BG361</t>
+          <t>BG362</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>BG361 PWCS Koorgang Bengalla</t>
+          <t>BG362 Bengalla PWCS Morandoo</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
@@ -14122,17 +14122,17 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>-32.28691</t>
+          <t>-32.279693</t>
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>150.83532</t>
+          <t>150.84704</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -14218,17 +14218,17 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>-32.343863</t>
+          <t>-32.353867</t>
         </is>
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>149.95028</t>
+          <t>150.097053</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -14266,17 +14266,17 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t>-32.353017</t>
+          <t>-32.402567</t>
         </is>
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>150.61636</t>
+          <t>150.364147</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -14362,17 +14362,17 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>-32.72273</t>
+          <t>-32.803257</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>151.494253</t>
+          <t>151.662773</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -14554,17 +14554,17 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
-          <t>-32.630813</t>
+          <t>-32.629653</t>
         </is>
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>151.11424</t>
+          <t>151.11664</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
@@ -18098,17 +18098,17 @@
       </c>
       <c r="G369" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H369" s="2" t="inlineStr">
         <is>
-          <t>-27.89897</t>
+          <t>-27.557003</t>
         </is>
       </c>
       <c r="I369" s="2" t="inlineStr">
         <is>
-          <t>152.925507</t>
+          <t>153.024347</t>
         </is>
       </c>
       <c r="J369" s="2" t="inlineStr">
@@ -18146,17 +18146,17 @@
       </c>
       <c r="G370" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H370" s="2" t="inlineStr">
         <is>
-          <t>-32.706647</t>
+          <t>-32.923587</t>
         </is>
       </c>
       <c r="I370" s="2" t="inlineStr">
         <is>
-          <t>151.542333</t>
+          <t>151.733893</t>
         </is>
       </c>
       <c r="J370" s="2" t="inlineStr">
@@ -18611,12 +18611,12 @@
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>ER408</t>
+          <t>MN409</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
         <is>
-          <t>ER408 Various Mines Eraring</t>
+          <t>MN409 Vales Point / Eraring Mangoola</t>
         </is>
       </c>
       <c r="F380" s="2" t="inlineStr">
@@ -18626,17 +18626,17 @@
       </c>
       <c r="G380" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T17:02:28.169445Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H380" s="2" t="inlineStr">
         <is>
-          <t>-32.943867</t>
+          <t>-33.04348</t>
         </is>
       </c>
       <c r="I380" s="2" t="inlineStr">
         <is>
-          <t>151.61816</t>
+          <t>151.524013</t>
         </is>
       </c>
       <c r="J380" s="2" t="inlineStr">
@@ -18659,12 +18659,12 @@
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>RV115</t>
+          <t>RV116</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>RV115 PWCS Kooragang Ravensworth</t>
+          <t>RV116 Ravensworth PWCS Kooragang</t>
         </is>
       </c>
       <c r="F381" s="2" t="inlineStr">
@@ -18674,17 +18674,17 @@
       </c>
       <c r="G381" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H381" s="2" t="inlineStr">
         <is>
-          <t>-32.4036</t>
+          <t>-32.40865</t>
         </is>
       </c>
       <c r="I381" s="2" t="inlineStr">
         <is>
-          <t>151.018347</t>
+          <t>151.022813</t>
         </is>
       </c>
       <c r="J381" s="2" t="inlineStr">
@@ -18722,17 +18722,17 @@
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H382" s="2" t="inlineStr">
         <is>
-          <t>-32.572497</t>
+          <t>-32.35278</t>
         </is>
       </c>
       <c r="I382" s="2" t="inlineStr">
         <is>
-          <t>151.166133</t>
+          <t>151.003853</t>
         </is>
       </c>
       <c r="J382" s="2" t="inlineStr">
@@ -18866,17 +18866,17 @@
       </c>
       <c r="G385" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H385" s="2" t="inlineStr">
         <is>
-          <t>-32.43212</t>
+          <t>-32.346057</t>
         </is>
       </c>
       <c r="I385" s="2" t="inlineStr">
         <is>
-          <t>150.211413</t>
+          <t>150.07096</t>
         </is>
       </c>
       <c r="J385" s="2" t="inlineStr">
@@ -18914,17 +18914,17 @@
       </c>
       <c r="G386" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H386" s="2" t="inlineStr">
         <is>
-          <t>-32.71318</t>
+          <t>-32.776143</t>
         </is>
       </c>
       <c r="I386" s="2" t="inlineStr">
         <is>
-          <t>151.409133</t>
+          <t>151.631</t>
         </is>
       </c>
       <c r="J386" s="2" t="inlineStr">
@@ -18962,17 +18962,17 @@
       </c>
       <c r="G387" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:02:51.535895Z</t>
+          <t>2026-05-02T18:33:10.010197Z</t>
         </is>
       </c>
       <c r="H387" s="2" t="inlineStr">
         <is>
-          <t>-32.739123</t>
+          <t>-32.836983</t>
         </is>
       </c>
       <c r="I387" s="2" t="inlineStr">
         <is>
-          <t>151.5744</t>
+          <t>151.687253</t>
         </is>
       </c>
       <c r="J387" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update RailOps database files - 2026-05-02 19:32:38 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_database.xlsx
+++ b/static/downloads/loco_database.xlsx
@@ -589,17 +589,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-33.733137</t>
+          <t>-33.552453</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>151.076973</t>
+          <t>151.197693</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -685,17 +685,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-33.91931</t>
+          <t>-33.9629</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>151.16732</t>
+          <t>151.219467</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-34.305187</t>
+          <t>-34.305353</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>150.59256</t>
+          <t>150.592827</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -821,17 +821,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-34.30561</t>
+          <t>-34.305713</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>150.594</t>
+          <t>150.594253</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>-30.999807</t>
+          <t>-31.01194</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>126.22424</t>
+          <t>125.704387</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2449,17 +2449,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>-34.18219</t>
+          <t>-34.181937</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>150.613413</t>
+          <t>150.613373</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2497,17 +2497,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>-34.184893</t>
+          <t>-34.184653</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>150.613733</t>
+          <t>150.61372</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2525,17 +2525,17 @@
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Empty Coal</t>
+          <t>PN Light Engine Movement</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>M542</t>
+          <t>D110</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>M542 Jilalan Yard / Callemondah Yard German Creek</t>
+          <t>D110</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2545,17 +2545,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T17:02:28.169445Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>-33.90311</t>
+          <t>-33.90159</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>150.937213</t>
+          <t>151.072333</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3165,17 +3165,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>-32.902973</t>
+          <t>-32.903003</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>151.755227</t>
+          <t>151.755093</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3261,17 +3261,17 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>-34.231583</t>
+          <t>-34.2209</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>150.58176</t>
+          <t>150.5912</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -3357,17 +3357,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>-31.346823</t>
+          <t>-31.48827</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>150.633933</t>
+          <t>150.68268</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3497,17 +3497,17 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>-30.968657</t>
+          <t>-30.968647</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>150.235267</t>
+          <t>150.23528</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3545,17 +3545,17 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>-32.341987</t>
+          <t>-32.392757</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>150.986053</t>
+          <t>151.031493</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>-31.349307</t>
+          <t>-31.3491</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>150.646107</t>
+          <t>150.646027</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3722,12 +3722,12 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>ND278</t>
+          <t>HV939</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>ND278 Newdell PWCS Kooragang</t>
+          <t>HV939 Port Waratah Hunter Valley</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>-32.867243</t>
+          <t>-32.863867</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>151.754347</t>
+          <t>151.727147</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>-32.872957</t>
+          <t>-32.86926</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>151.739253</t>
+          <t>151.72156</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3833,17 +3833,17 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>-31.642917</t>
+          <t>-31.692</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>150.720187</t>
+          <t>150.7688</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3929,17 +3929,17 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>-30.99344</t>
+          <t>-30.967007</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>150.278933</t>
+          <t>150.23084</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3977,17 +3977,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-32.671557</t>
+          <t>-32.671357</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>151.370293</t>
+          <t>151.370413</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4073,17 +4073,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>-32.46114</t>
+          <t>-32.616913</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>151.106547</t>
+          <t>151.215587</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4121,17 +4121,17 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>-32.39081</t>
+          <t>-32.45829</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>151.030707</t>
+          <t>151.070973</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -4169,17 +4169,17 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>-32.803293</t>
+          <t>-32.836863</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>151.662827</t>
+          <t>151.68724</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4265,17 +4265,17 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>-30.774113</t>
+          <t>-30.821647</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>128.897787</t>
+          <t>128.412227</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4453,12 +4453,12 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>-30.778048</t>
+          <t>-30.778067</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -4549,17 +4549,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>-32.879667</t>
+          <t>-32.90822</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>143.931067</t>
+          <t>144.243613</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4645,17 +4645,17 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>-33.240687</t>
+          <t>-33.019917</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>138.12248</t>
+          <t>138.01112</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4693,17 +4693,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>-30.58177</t>
+          <t>-30.554553</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>130.687453</t>
+          <t>130.92044</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -4789,17 +4789,17 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>-30.781407</t>
+          <t>-30.841277</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>121.415307</t>
+          <t>121.192307</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4837,17 +4837,17 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>-37.082173</t>
+          <t>-36.947867</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>142.797227</t>
+          <t>142.688893</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4933,12 +4933,12 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>-36.645153</t>
+          <t>-36.645147</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -4981,17 +4981,17 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>-32.36749</t>
+          <t>-32.04842</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>137.62468</t>
+          <t>137.401093</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -5029,17 +5029,17 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>-31.020213</t>
+          <t>-31.03231</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>123.076667</t>
+          <t>123.592573</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5221,17 +5221,17 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:33:10.010197Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>-34.809973</t>
+          <t>-34.765253</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>138.605987</t>
+          <t>138.64224</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -5505,17 +5505,17 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>-36.79731</t>
+          <t>-36.87285</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>142.58244</t>
+          <t>142.63612</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -5601,17 +5601,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>-32.179743</t>
+          <t>-32.060283</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>148.630373</t>
+          <t>148.666787</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5634,12 +5634,12 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>8178</t>
+          <t>1877</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>8178 Grainforce Siding, Kelso Port Botany</t>
+          <t>1877 Port Botany Grainforce Siding, Kelso</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -5649,17 +5649,17 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>-33.95874</t>
+          <t>-33.949047</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>151.219</t>
+          <t>151.213</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -5793,17 +5793,17 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>-33.10407</t>
+          <t>-33.10467</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>149.9974</t>
+          <t>149.995347</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>-33.732603</t>
+          <t>-33.552577</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>151.077507</t>
+          <t>151.197547</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -6081,17 +6081,17 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>-30.892793</t>
+          <t>-30.870683</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>120.871067</t>
+          <t>120.59576</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -6129,17 +6129,17 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>-33.602937</t>
+          <t>-33.901313</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>138.225</t>
+          <t>138.229893</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -6225,17 +6225,17 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>-30.662843</t>
+          <t>-30.96929</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>150.02208</t>
+          <t>150.235707</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6513,17 +6513,17 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>-37.160087</t>
+          <t>-37.382537</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>142.86008</t>
+          <t>142.92176</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -6561,17 +6561,17 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>-31.544317</t>
+          <t>-31.48415</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>118.019933</t>
+          <t>118.294907</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -6609,17 +6609,17 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>-31.21467</t>
+          <t>-31.16566</t>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>136.330933</t>
+          <t>136.125173</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -6946,17 +6946,17 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>-33.90368</t>
+          <t>-33.90367</t>
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>151.073987</t>
+          <t>151.074027</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -7022,17 +7022,17 @@
       <c r="B138" s="2" t="inlineStr"/>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>SSR Loaded Cement</t>
+          <t>SSR Empty Cement</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>4645</t>
+          <t>6244</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>4645 Broadmeadow Boambee Beach</t>
+          <t>6244 Boambee Beach Berrima Cement Works</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -7042,17 +7042,17 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T08:03:36.971806Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>-30.315843</t>
+          <t>-30.31472</t>
         </is>
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>153.131667</t>
+          <t>153.1332</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -7090,17 +7090,17 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>-33.949803</t>
+          <t>-33.910393</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>151.213653</t>
+          <t>151.102947</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -7618,17 +7618,17 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T17:33:30.507033Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>-23.656</t>
+          <t>-23.696693</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>133.85084</t>
+          <t>133.872613</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -7666,17 +7666,17 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>-23.691195</t>
+          <t>-23.688088</t>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>133.864013</t>
+          <t>133.8592</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -7714,17 +7714,17 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>-29.76529</t>
+          <t>-29.304127</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>134.539173</t>
+          <t>134.525653</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -7795,12 +7795,12 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>1122</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>1122 Pelican Point/Port Flat Dry Creek North</t>
+          <t>1120 Pelican Point/Port Flat Dry Creek North</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -7810,17 +7810,17 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>-34.786953</t>
+          <t>-34.820563</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>138.5042</t>
+          <t>138.596893</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -7858,17 +7858,17 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>-14.230667</t>
+          <t>-14.504883</t>
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>132.05476</t>
+          <t>132.243093</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -7906,17 +7906,17 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>-31.221337</t>
+          <t>-31.23142</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>136.461627</t>
+          <t>136.667453</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>-34.308013</t>
+          <t>-34.563703</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>138.358947</t>
+          <t>138.513067</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -8002,17 +8002,17 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>-32.723367</t>
+          <t>-32.79806</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>151.496293</t>
+          <t>151.656707</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -8050,17 +8050,17 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>-32.86967</t>
+          <t>-32.867883</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>151.758027</t>
+          <t>151.753707</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -8098,17 +8098,17 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>-32.37135</t>
+          <t>-32.408607</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>150.476307</t>
+          <t>150.64592</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -8146,17 +8146,17 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>-32.663683</t>
+          <t>-32.730257</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>151.313573</t>
+          <t>151.531493</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -8366,17 +8366,17 @@
       <c r="B166" s="2" t="inlineStr"/>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Hunter Line Service</t>
+          <t>Empty Car Transfer</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>V792</t>
+          <t>V813</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>V792 Telarah Newcastle Interchange</t>
+          <t>V813 Broadmeadow Yard Newcastle Interchange</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -8386,17 +8386,17 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01T16:33:33.123186Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>-32.92212</t>
+          <t>-32.92305</t>
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>151.754547</t>
+          <t>151.756653</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -8578,17 +8578,17 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>-32.637983</t>
+          <t>-32.318283</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>151.227053</t>
+          <t>150.978387</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -8722,17 +8722,17 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>-32.923877</t>
+          <t>-32.751067</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>151.7586</t>
+          <t>151.594013</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -8958,17 +8958,17 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>-32.872953</t>
+          <t>-32.873753</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>151.747267</t>
+          <t>151.741107</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -9006,17 +9006,17 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>-32.390933</t>
+          <t>-32.388553</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>150.995693</t>
+          <t>150.996613</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -9054,17 +9054,17 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>-32.602733</t>
+          <t>-32.632163</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>151.19876</t>
+          <t>151.102813</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
@@ -9102,17 +9102,17 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>-33.51585</t>
+          <t>-33.502807</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>150.011213</t>
+          <t>149.748227</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -9198,17 +9198,17 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>-33.48055</t>
+          <t>-33.405</t>
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>150.1574</t>
+          <t>150.080533</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -9530,17 +9530,17 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>-33.890737</t>
+          <t>-33.866613</t>
         </is>
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>151.067933</t>
+          <t>151.060027</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
@@ -9578,17 +9578,17 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T15:34:12.020596Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
-          <t>-29.50484</t>
+          <t>-29.502567</t>
         </is>
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>149.853293</t>
+          <t>149.853387</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr">
@@ -10054,17 +10054,17 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>-35.215647</t>
+          <t>-35.254807</t>
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>139.418947</t>
+          <t>139.456107</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
@@ -10294,17 +10294,17 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>-31.089793</t>
+          <t>-30.947843</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>135.890707</t>
+          <t>135.433893</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
@@ -10486,12 +10486,12 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>-32.46907</t>
+          <t>-32.469077</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
@@ -10534,17 +10534,17 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>-30.912963</t>
+          <t>-30.871147</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>120.81392</t>
+          <t>121.071107</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr">
@@ -10582,17 +10582,17 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>-32.585733</t>
+          <t>-32.721463</t>
         </is>
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>142.928747</t>
+          <t>143.258133</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr">
@@ -10678,17 +10678,17 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>-33.083063</t>
+          <t>-33.017077</t>
         </is>
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>147.15612</t>
+          <t>146.70732</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -10774,17 +10774,17 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>-31.004347</t>
+          <t>-31.03248</t>
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>135.59736</t>
+          <t>135.725573</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -10822,17 +10822,17 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>-30.579217</t>
+          <t>-30.61229</t>
         </is>
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>130.708867</t>
+          <t>130.419667</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
@@ -10870,17 +10870,17 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>-32.888807</t>
+          <t>-32.716227</t>
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>151.71136</t>
+          <t>151.544707</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr">
@@ -10918,17 +10918,17 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>-31.526217</t>
+          <t>-31.59228</t>
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>118.090707</t>
+          <t>117.927293</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr">
@@ -10966,17 +10966,17 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>-30.720013</t>
+          <t>-30.950907</t>
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>152.91372</t>
+          <t>152.851893</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
@@ -11014,17 +11014,17 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t>-30.61283</t>
+          <t>-30.612833</t>
         </is>
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>130.415627</t>
+          <t>130.41564</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -11110,17 +11110,17 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t>-30.742447</t>
+          <t>-30.740783</t>
         </is>
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>121.470627</t>
+          <t>121.516493</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -11254,17 +11254,17 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t>-32.381643</t>
+          <t>-32.186713</t>
         </is>
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>140.11944</t>
+          <t>140.583493</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr">
@@ -11638,17 +11638,17 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>-33.093973</t>
+          <t>-32.943173</t>
         </is>
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>151.49696</t>
+          <t>151.6692</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr">
@@ -11686,17 +11686,17 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>-30.88603</t>
+          <t>-30.731437</t>
         </is>
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>121.802653</t>
+          <t>121.50512</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr">
@@ -11734,17 +11734,17 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>-30.684077</t>
+          <t>-30.707953</t>
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>134.22448</t>
+          <t>134.602027</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr">
@@ -11782,17 +11782,17 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
-          <t>-33.036187</t>
+          <t>-33.04237</t>
         </is>
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>145.547613</t>
+          <t>145.17272</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr">
@@ -11878,17 +11878,17 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
-          <t>-35.51969</t>
+          <t>-35.189153</t>
         </is>
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>139.766587</t>
+          <t>139.390213</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
@@ -12098,17 +12098,17 @@
       <c r="B244" s="2" t="inlineStr"/>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Watco Trip Train</t>
+          <t>Watco Light Engine</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>T922</t>
+          <t>D921</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>T922</t>
+          <t>D921</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
@@ -12118,17 +12118,17 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>-34.457177</t>
+          <t>-34.463497</t>
         </is>
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>150.87624</t>
+          <t>150.87744</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr">
@@ -12306,17 +12306,17 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>-28.937981</t>
+          <t>-29.003584</t>
         </is>
       </c>
       <c r="I248" s="2" t="inlineStr">
         <is>
-          <t>121.516686</t>
+          <t>121.500923</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr">
@@ -12354,17 +12354,17 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
-          <t>-30.777277</t>
+          <t>-30.777294</t>
         </is>
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>121.422928</t>
+          <t>121.422905</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr">
@@ -12690,17 +12690,17 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
-          <t>-31.52426</t>
+          <t>-31.50729</t>
         </is>
       </c>
       <c r="I256" s="2" t="inlineStr">
         <is>
-          <t>146.16644</t>
+          <t>145.929</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr">
@@ -12786,17 +12786,17 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
-          <t>-33.005</t>
+          <t>-33.2969</t>
         </is>
       </c>
       <c r="I258" s="2" t="inlineStr">
         <is>
-          <t>151.5548</t>
+          <t>151.422693</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr">
@@ -13162,17 +13162,17 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>-33.186767</t>
+          <t>-33.18677</t>
         </is>
       </c>
       <c r="I266" s="2" t="inlineStr">
         <is>
-          <t>148.695</t>
+          <t>148.694627</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr">
@@ -13210,17 +13210,17 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01T19:31:30.048631Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>-33.964697</t>
+          <t>-33.859867</t>
         </is>
       </c>
       <c r="I267" s="2" t="inlineStr">
         <is>
-          <t>151.218933</t>
+          <t>150.972187</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr">
@@ -13258,17 +13258,17 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>-32.61443</t>
+          <t>-32.596037</t>
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr">
         <is>
-          <t>143.011413</t>
+          <t>142.95848</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr">
@@ -13354,17 +13354,17 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr">
         <is>
-          <t>-30.765993</t>
+          <t>-30.722393</t>
         </is>
       </c>
       <c r="I270" s="2" t="inlineStr">
         <is>
-          <t>128.97948</t>
+          <t>129.405133</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr">
@@ -13402,17 +13402,17 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
         <is>
-          <t>-23.607254</t>
+          <t>-23.564893</t>
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr">
         <is>
-          <t>148.519262</t>
+          <t>148.29865</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr">
@@ -13786,17 +13786,17 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
         <is>
-          <t>-32.4221</t>
+          <t>-32.499413</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>151.0506</t>
+          <t>151.137747</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -13834,17 +13834,17 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>-32.289027</t>
+          <t>-32.286573</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>150.822773</t>
+          <t>150.824187</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -13978,17 +13978,17 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t>-32.46633</t>
+          <t>-32.595403</t>
         </is>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>151.119107</t>
+          <t>151.191867</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
@@ -14074,17 +14074,17 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>-32.873347</t>
+          <t>-32.870673</t>
         </is>
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>151.768427</t>
+          <t>151.76244</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
@@ -14122,17 +14122,17 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>-32.28024</t>
+          <t>-32.346907</t>
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>150.91908</t>
+          <t>150.988227</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
@@ -14170,17 +14170,17 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
-          <t>-32.864703</t>
+          <t>-32.77083</t>
         </is>
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>151.740507</t>
+          <t>151.624693</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
@@ -14218,17 +14218,17 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>-32.437427</t>
+          <t>-32.423173</t>
         </is>
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>150.148333</t>
+          <t>150.27536</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
@@ -14266,17 +14266,17 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t>-32.423833</t>
+          <t>-32.345993</t>
         </is>
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>150.13148</t>
+          <t>149.951787</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
@@ -14314,17 +14314,17 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>-30.62882</t>
+          <t>-30.770003</t>
         </is>
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>150.05592</t>
+          <t>150.042107</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -14362,17 +14362,17 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>-32.86607</t>
+          <t>-32.874917</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>151.749707</t>
+          <t>151.771507</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
@@ -14410,17 +14410,17 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>-32.665167</t>
+          <t>-32.472223</t>
         </is>
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>151.35548</t>
+          <t>151.12884</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
@@ -18194,17 +18194,17 @@
       </c>
       <c r="G371" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H371" s="2" t="inlineStr">
         <is>
-          <t>-33.11067</t>
+          <t>-33.449827</t>
         </is>
       </c>
       <c r="I371" s="2" t="inlineStr">
         <is>
-          <t>151.485467</t>
+          <t>151.322187</t>
         </is>
       </c>
       <c r="J371" s="2" t="inlineStr">
@@ -18366,17 +18366,17 @@
       <c r="B375" s="2" t="inlineStr"/>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>NSW Trainlink Empty Car Transfer</t>
+          <t>NSW TrainLink XPT</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>HT47</t>
+          <t>NT36</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
         <is>
-          <t>HT47</t>
+          <t>NT36 Grafton Central</t>
         </is>
       </c>
       <c r="F375" s="2" t="inlineStr">
@@ -18386,17 +18386,17 @@
       </c>
       <c r="G375" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T01:33:05.355076Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H375" s="2" t="inlineStr">
         <is>
-          <t>-33.85794</t>
+          <t>-29.828727</t>
         </is>
       </c>
       <c r="I375" s="2" t="inlineStr">
         <is>
-          <t>151.087853</t>
+          <t>152.98756</t>
         </is>
       </c>
       <c r="J375" s="2" t="inlineStr">
@@ -18515,12 +18515,12 @@
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>HT13</t>
+          <t>HT11</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
         <is>
-          <t>HT13</t>
+          <t>HT11</t>
         </is>
       </c>
       <c r="F378" s="2" t="inlineStr">
@@ -18530,17 +18530,17 @@
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T11:02:54.863060Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
         <is>
-          <t>-33.843997</t>
+          <t>-33.91513</t>
         </is>
       </c>
       <c r="I378" s="2" t="inlineStr">
         <is>
-          <t>151.085267</t>
+          <t>151.16572</t>
         </is>
       </c>
       <c r="J378" s="2" t="inlineStr">
@@ -18674,17 +18674,17 @@
       </c>
       <c r="G381" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T18:33:10.010197Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H381" s="2" t="inlineStr">
         <is>
-          <t>-33.04348</t>
+          <t>-32.89581</t>
         </is>
       </c>
       <c r="I381" s="2" t="inlineStr">
         <is>
-          <t>151.524013</t>
+          <t>151.724133</t>
         </is>
       </c>
       <c r="J381" s="2" t="inlineStr">
@@ -18722,17 +18722,17 @@
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H382" s="2" t="inlineStr">
         <is>
-          <t>-32.434777</t>
+          <t>-32.53998</t>
         </is>
       </c>
       <c r="I382" s="2" t="inlineStr">
         <is>
-          <t>151.05592</t>
+          <t>151.155653</t>
         </is>
       </c>
       <c r="J382" s="2" t="inlineStr">
@@ -18770,17 +18770,17 @@
       </c>
       <c r="G383" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H383" s="2" t="inlineStr">
         <is>
-          <t>-32.329513</t>
+          <t>-32.335133</t>
         </is>
       </c>
       <c r="I383" s="2" t="inlineStr">
         <is>
-          <t>150.894693</t>
+          <t>150.900907</t>
         </is>
       </c>
       <c r="J383" s="2" t="inlineStr">
@@ -18818,17 +18818,17 @@
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H384" s="2" t="inlineStr">
         <is>
-          <t>-32.85359</t>
+          <t>-32.711357</t>
         </is>
       </c>
       <c r="I384" s="2" t="inlineStr">
         <is>
-          <t>151.694627</t>
+          <t>151.408093</t>
         </is>
       </c>
       <c r="J384" s="2" t="inlineStr">
@@ -18914,17 +18914,17 @@
       </c>
       <c r="G386" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H386" s="2" t="inlineStr">
         <is>
-          <t>-32.314837</t>
+          <t>-32.273473</t>
         </is>
       </c>
       <c r="I386" s="2" t="inlineStr">
         <is>
-          <t>149.8596</t>
+          <t>149.759533</t>
         </is>
       </c>
       <c r="J386" s="2" t="inlineStr">
@@ -18962,17 +18962,17 @@
       </c>
       <c r="G387" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H387" s="2" t="inlineStr">
         <is>
-          <t>-32.878903</t>
+          <t>-32.875017</t>
         </is>
       </c>
       <c r="I387" s="2" t="inlineStr">
         <is>
-          <t>151.708213</t>
+          <t>151.77136</t>
         </is>
       </c>
       <c r="J387" s="2" t="inlineStr">
@@ -19010,17 +19010,17 @@
       </c>
       <c r="G388" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T19:02:52.469359Z</t>
+          <t>2026-05-02T19:32:38.436985Z</t>
         </is>
       </c>
       <c r="H388" s="2" t="inlineStr">
         <is>
-          <t>-32.837007</t>
+          <t>-32.836983</t>
         </is>
       </c>
       <c r="I388" s="2" t="inlineStr">
         <is>
-          <t>151.68724</t>
+          <t>151.687253</t>
         </is>
       </c>
       <c r="J388" s="2" t="inlineStr">

</xml_diff>